<commit_message>
feat: add snowflake impl
</commit_message>
<xml_diff>
--- a/docs/result.xlsx
+++ b/docs/result.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/muhammadrayandika/projects/bmkg_weather_forecasting/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{312B65A8-D0F4-4E48-B182-7E8B39E554F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C768A098-3E72-9E46-9ED4-66E582A02DFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13080" yWindow="-20900" windowWidth="19100" windowHeight="20880" xr2:uid="{5AC5918A-7EFC-C743-9AF6-45D314C9895F}"/>
+    <workbookView xWindow="0" yWindow="700" windowWidth="33600" windowHeight="20280" activeTab="1" xr2:uid="{5AC5918A-7EFC-C743-9AF6-45D314C9895F}"/>
   </bookViews>
   <sheets>
-    <sheet name="Result Of Optimization ETL" sheetId="1" r:id="rId1"/>
+    <sheet name="Result Starflake" sheetId="1" r:id="rId1"/>
+    <sheet name="Result Snowflake" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="15">
   <si>
     <t>Percobaan 1</t>
   </si>
@@ -69,6 +70,18 @@
   <si>
     <t>Satuan Dalam bentuk : mili second (ms)</t>
   </si>
+  <si>
+    <t>Snowflake Sebelum Optimasi</t>
+  </si>
+  <si>
+    <t>Snowflake Sesudah Optimasi ( Subquery, Indexing, dan Partition)</t>
+  </si>
+  <si>
+    <t>Snowflake Sesudah Optimasi ( Pararel Execution, Indexing dan Partition)</t>
+  </si>
+  <si>
+    <t>Snowflake Sesudah Optimasi ( Kombinasi : Pararel Execution, Subindexing dan partitioning)</t>
+  </si>
 </sst>
 </file>
 
@@ -79,7 +92,7 @@
     <numFmt numFmtId="164" formatCode="#,##0.000"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -101,8 +114,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -127,8 +147,26 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -151,20 +189,54 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -176,7 +248,31 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="3" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -536,22 +632,22 @@
       <c r="P3" s="9"/>
     </row>
     <row r="6" spans="5:19" x14ac:dyDescent="0.2">
-      <c r="E6" s="3" t="s">
+      <c r="E6" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
-      <c r="I6" s="3"/>
-      <c r="J6" s="3"/>
-      <c r="N6" s="3" t="s">
+      <c r="F6" s="8"/>
+      <c r="G6" s="8"/>
+      <c r="H6" s="8"/>
+      <c r="I6" s="8"/>
+      <c r="J6" s="8"/>
+      <c r="N6" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="O6" s="3"/>
-      <c r="P6" s="3"/>
-      <c r="Q6" s="3"/>
-      <c r="R6" s="3"/>
-      <c r="S6" s="3"/>
+      <c r="O6" s="8"/>
+      <c r="P6" s="8"/>
+      <c r="Q6" s="8"/>
+      <c r="R6" s="8"/>
+      <c r="S6" s="8"/>
     </row>
     <row r="8" spans="5:19" x14ac:dyDescent="0.2">
       <c r="F8" s="2">
@@ -589,10 +685,10 @@
       <c r="E9" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="F9" s="4">
+      <c r="F9" s="3">
         <v>111.376</v>
       </c>
-      <c r="G9" s="5">
+      <c r="G9" s="4">
         <v>143.88900000000001</v>
       </c>
       <c r="H9" s="1">
@@ -607,19 +703,19 @@
       <c r="N9" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="O9" s="8">
+      <c r="O9" s="7">
         <v>77.754999999999995</v>
       </c>
-      <c r="P9" s="8">
+      <c r="P9" s="7">
         <v>119.75700000000001</v>
       </c>
-      <c r="Q9" s="8">
+      <c r="Q9" s="7">
         <v>165.14099999999999</v>
       </c>
-      <c r="R9" s="8">
+      <c r="R9" s="7">
         <v>229.625</v>
       </c>
-      <c r="S9" s="8">
+      <c r="S9" s="7">
         <v>308.29300000000001</v>
       </c>
     </row>
@@ -627,10 +723,10 @@
       <c r="E10" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="F10" s="4">
+      <c r="F10" s="3">
         <v>112.614</v>
       </c>
-      <c r="G10" s="5">
+      <c r="G10" s="4">
         <v>136.73699999999999</v>
       </c>
       <c r="H10" s="1">
@@ -645,19 +741,19 @@
       <c r="N10" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="O10" s="8">
+      <c r="O10" s="7">
         <v>76.718999999999994</v>
       </c>
-      <c r="P10" s="8">
+      <c r="P10" s="7">
         <v>99.938999999999993</v>
       </c>
-      <c r="Q10" s="8">
+      <c r="Q10" s="7">
         <v>190.42500000000001</v>
       </c>
-      <c r="R10" s="8">
+      <c r="R10" s="7">
         <v>239.77799999999999</v>
       </c>
-      <c r="S10" s="8">
+      <c r="S10" s="7">
         <v>275.48099999999999</v>
       </c>
     </row>
@@ -665,10 +761,10 @@
       <c r="E11" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="F11" s="4">
+      <c r="F11" s="3">
         <v>128.07599999999999</v>
       </c>
-      <c r="G11" s="5">
+      <c r="G11" s="4">
         <v>213.71899999999999</v>
       </c>
       <c r="H11" s="1">
@@ -683,19 +779,19 @@
       <c r="N11" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="O11" s="8">
+      <c r="O11" s="7">
         <v>140.524</v>
       </c>
-      <c r="P11" s="8">
+      <c r="P11" s="7">
         <v>97.105999999999995</v>
       </c>
-      <c r="Q11" s="8">
+      <c r="Q11" s="7">
         <v>208.499</v>
       </c>
-      <c r="R11" s="8">
+      <c r="R11" s="7">
         <v>242.53899999999999</v>
       </c>
-      <c r="S11" s="8">
+      <c r="S11" s="7">
         <v>228.61699999999999</v>
       </c>
     </row>
@@ -703,10 +799,10 @@
       <c r="E12" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="F12" s="4">
+      <c r="F12" s="3">
         <v>182.779</v>
       </c>
-      <c r="G12" s="5">
+      <c r="G12" s="4">
         <v>138.977</v>
       </c>
       <c r="H12" s="1">
@@ -721,19 +817,19 @@
       <c r="N12" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="O12" s="8">
+      <c r="O12" s="7">
         <v>97.156000000000006</v>
       </c>
-      <c r="P12" s="8">
+      <c r="P12" s="7">
         <v>99.393000000000001</v>
       </c>
-      <c r="Q12" s="8">
+      <c r="Q12" s="7">
         <v>172.39699999999999</v>
       </c>
-      <c r="R12" s="8">
+      <c r="R12" s="7">
         <v>278.01600000000002</v>
       </c>
-      <c r="S12" s="8">
+      <c r="S12" s="7">
         <v>233.97800000000001</v>
       </c>
     </row>
@@ -741,10 +837,10 @@
       <c r="E13" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F13" s="4">
+      <c r="F13" s="3">
         <v>109.913</v>
       </c>
-      <c r="G13" s="5">
+      <c r="G13" s="4">
         <v>140.35400000000001</v>
       </c>
       <c r="H13" s="1">
@@ -759,79 +855,79 @@
       <c r="N13" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="O13" s="8">
+      <c r="O13" s="7">
         <v>77.403000000000006</v>
       </c>
-      <c r="P13" s="8">
+      <c r="P13" s="7">
         <v>103.63500000000001</v>
       </c>
-      <c r="Q13" s="8">
+      <c r="Q13" s="7">
         <v>159.054</v>
       </c>
-      <c r="R13" s="8">
+      <c r="R13" s="7">
         <v>240.28299999999999</v>
       </c>
-      <c r="S13" s="8">
+      <c r="S13" s="7">
         <v>249.54400000000001</v>
       </c>
     </row>
     <row r="14" spans="5:19" x14ac:dyDescent="0.2">
-      <c r="E14" s="6" t="s">
+      <c r="E14" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="F14" s="7">
+      <c r="F14" s="6">
         <f>AVERAGE(F9:F13)</f>
         <v>128.95160000000001</v>
       </c>
-      <c r="G14" s="7">
+      <c r="G14" s="6">
         <f t="shared" ref="G14:J14" si="0">AVERAGE(G9:G13)</f>
         <v>154.73520000000002</v>
       </c>
-      <c r="H14" s="7">
+      <c r="H14" s="6">
         <f t="shared" si="0"/>
         <v>310.47000000000003</v>
       </c>
-      <c r="I14" s="7">
+      <c r="I14" s="6">
         <f t="shared" si="0"/>
         <v>353.55399999999997</v>
       </c>
-      <c r="J14" s="7">
+      <c r="J14" s="6">
         <f t="shared" si="0"/>
         <v>377.14640000000003</v>
       </c>
-      <c r="N14" s="6" t="s">
+      <c r="N14" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="O14" s="7">
+      <c r="O14" s="6">
         <f>AVERAGE(O9:O13)</f>
         <v>93.9114</v>
       </c>
-      <c r="P14" s="7">
+      <c r="P14" s="6">
         <f t="shared" ref="P14" si="1">AVERAGE(P9:P13)</f>
         <v>103.96600000000001</v>
       </c>
-      <c r="Q14" s="7">
+      <c r="Q14" s="6">
         <f t="shared" ref="Q14" si="2">AVERAGE(Q9:Q13)</f>
         <v>179.10319999999999</v>
       </c>
-      <c r="R14" s="7">
+      <c r="R14" s="6">
         <f t="shared" ref="R14" si="3">AVERAGE(R9:R13)</f>
         <v>246.04820000000001</v>
       </c>
-      <c r="S14" s="7">
+      <c r="S14" s="6">
         <f t="shared" ref="S14" si="4">AVERAGE(S9:S13)</f>
         <v>259.18259999999998</v>
       </c>
     </row>
     <row r="20" spans="14:19" x14ac:dyDescent="0.2">
-      <c r="N20" s="3" t="s">
+      <c r="N20" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="O20" s="3"/>
-      <c r="P20" s="3"/>
-      <c r="Q20" s="3"/>
-      <c r="R20" s="3"/>
-      <c r="S20" s="3"/>
+      <c r="O20" s="8"/>
+      <c r="P20" s="8"/>
+      <c r="Q20" s="8"/>
+      <c r="R20" s="8"/>
+      <c r="S20" s="8"/>
     </row>
     <row r="22" spans="14:19" x14ac:dyDescent="0.2">
       <c r="O22" s="2">
@@ -854,19 +950,19 @@
       <c r="N23" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="O23" s="8">
+      <c r="O23" s="7">
         <v>75.866</v>
       </c>
-      <c r="P23" s="8">
+      <c r="P23" s="7">
         <v>130.58199999999999</v>
       </c>
-      <c r="Q23" s="8">
+      <c r="Q23" s="7">
         <v>152.541</v>
       </c>
-      <c r="R23" s="8">
+      <c r="R23" s="7">
         <v>249.38900000000001</v>
       </c>
-      <c r="S23" s="8">
+      <c r="S23" s="7">
         <v>232.51900000000001</v>
       </c>
     </row>
@@ -874,19 +970,19 @@
       <c r="N24" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="O24" s="8">
+      <c r="O24" s="7">
         <v>94.698999999999998</v>
       </c>
-      <c r="P24" s="8">
+      <c r="P24" s="7">
         <v>99.510999999999996</v>
       </c>
-      <c r="Q24" s="8">
+      <c r="Q24" s="7">
         <v>184.23699999999999</v>
       </c>
-      <c r="R24" s="8">
+      <c r="R24" s="7">
         <v>255.25399999999999</v>
       </c>
-      <c r="S24" s="8">
+      <c r="S24" s="7">
         <v>265.57600000000002</v>
       </c>
     </row>
@@ -894,19 +990,19 @@
       <c r="N25" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="O25" s="8">
+      <c r="O25" s="7">
         <v>102.77</v>
       </c>
-      <c r="P25" s="8">
+      <c r="P25" s="7">
         <v>100.2</v>
       </c>
-      <c r="Q25" s="8">
+      <c r="Q25" s="7">
         <v>175.64099999999999</v>
       </c>
-      <c r="R25" s="8">
+      <c r="R25" s="7">
         <v>230.971</v>
       </c>
-      <c r="S25" s="8">
+      <c r="S25" s="7">
         <v>270.988</v>
       </c>
     </row>
@@ -914,19 +1010,19 @@
       <c r="N26" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="O26" s="8">
+      <c r="O26" s="7">
         <v>78.587000000000003</v>
       </c>
-      <c r="P26" s="8">
+      <c r="P26" s="7">
         <v>114.334</v>
       </c>
-      <c r="Q26" s="8">
+      <c r="Q26" s="7">
         <v>210.39599999999999</v>
       </c>
-      <c r="R26" s="8">
+      <c r="R26" s="7">
         <v>261.68400000000003</v>
       </c>
-      <c r="S26" s="8">
+      <c r="S26" s="7">
         <v>242.14</v>
       </c>
     </row>
@@ -934,56 +1030,56 @@
       <c r="N27" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="O27" s="8">
+      <c r="O27" s="7">
         <v>87.555000000000007</v>
       </c>
-      <c r="P27" s="8">
+      <c r="P27" s="7">
         <v>110.733</v>
       </c>
-      <c r="Q27" s="8">
+      <c r="Q27" s="7">
         <v>160.60300000000001</v>
       </c>
-      <c r="R27" s="8">
+      <c r="R27" s="7">
         <v>240.37</v>
       </c>
-      <c r="S27" s="8">
+      <c r="S27" s="7">
         <v>245.50899999999999</v>
       </c>
     </row>
     <row r="28" spans="14:19" x14ac:dyDescent="0.2">
-      <c r="N28" s="6" t="s">
+      <c r="N28" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="O28" s="7">
+      <c r="O28" s="6">
         <f>AVERAGE(O23:O27)</f>
         <v>87.895399999999995</v>
       </c>
-      <c r="P28" s="7">
+      <c r="P28" s="6">
         <f t="shared" ref="P28" si="5">AVERAGE(P23:P27)</f>
         <v>111.072</v>
       </c>
-      <c r="Q28" s="7">
+      <c r="Q28" s="6">
         <f t="shared" ref="Q28" si="6">AVERAGE(Q23:Q27)</f>
         <v>176.68359999999998</v>
       </c>
-      <c r="R28" s="7">
+      <c r="R28" s="6">
         <f t="shared" ref="R28" si="7">AVERAGE(R23:R27)</f>
         <v>247.53360000000004</v>
       </c>
-      <c r="S28" s="7">
+      <c r="S28" s="6">
         <f t="shared" ref="S28" si="8">AVERAGE(S23:S27)</f>
         <v>251.34639999999999</v>
       </c>
     </row>
     <row r="31" spans="14:19" x14ac:dyDescent="0.2">
-      <c r="N31" s="3" t="s">
+      <c r="N31" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="O31" s="3"/>
-      <c r="P31" s="3"/>
-      <c r="Q31" s="3"/>
-      <c r="R31" s="3"/>
-      <c r="S31" s="3"/>
+      <c r="O31" s="8"/>
+      <c r="P31" s="8"/>
+      <c r="Q31" s="8"/>
+      <c r="R31" s="8"/>
+      <c r="S31" s="8"/>
     </row>
     <row r="33" spans="14:19" x14ac:dyDescent="0.2">
       <c r="O33" s="2">
@@ -1006,19 +1102,19 @@
       <c r="N34" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="O34" s="8">
+      <c r="O34" s="7">
         <v>55.804000000000002</v>
       </c>
-      <c r="P34" s="8">
+      <c r="P34" s="7">
         <v>50.383000000000003</v>
       </c>
-      <c r="Q34" s="8">
+      <c r="Q34" s="7">
         <v>51.292999999999999</v>
       </c>
-      <c r="R34" s="8">
+      <c r="R34" s="7">
         <v>52.933999999999997</v>
       </c>
-      <c r="S34" s="8">
+      <c r="S34" s="7">
         <v>52.692999999999998</v>
       </c>
     </row>
@@ -1026,19 +1122,19 @@
       <c r="N35" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="O35" s="8">
+      <c r="O35" s="7">
         <v>65.367999999999995</v>
       </c>
-      <c r="P35" s="8">
+      <c r="P35" s="7">
         <v>69.436999999999998</v>
       </c>
-      <c r="Q35" s="8">
+      <c r="Q35" s="7">
         <v>51.094999999999999</v>
       </c>
-      <c r="R35" s="8">
+      <c r="R35" s="7">
         <v>52.177</v>
       </c>
-      <c r="S35" s="8">
+      <c r="S35" s="7">
         <v>58.481000000000002</v>
       </c>
     </row>
@@ -1046,19 +1142,19 @@
       <c r="N36" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="O36" s="8">
+      <c r="O36" s="7">
         <v>56.311</v>
       </c>
-      <c r="P36" s="8">
+      <c r="P36" s="7">
         <v>53.951999999999998</v>
       </c>
-      <c r="Q36" s="8">
+      <c r="Q36" s="7">
         <v>52.320999999999998</v>
       </c>
-      <c r="R36" s="8">
+      <c r="R36" s="7">
         <v>65.504000000000005</v>
       </c>
-      <c r="S36" s="8">
+      <c r="S36" s="7">
         <v>64.885000000000005</v>
       </c>
     </row>
@@ -1066,19 +1162,19 @@
       <c r="N37" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="O37" s="8">
+      <c r="O37" s="7">
         <v>63.237000000000002</v>
       </c>
-      <c r="P37" s="8">
+      <c r="P37" s="7">
         <v>51.546999999999997</v>
       </c>
-      <c r="Q37" s="8">
+      <c r="Q37" s="7">
         <v>53.494</v>
       </c>
-      <c r="R37" s="8">
+      <c r="R37" s="7">
         <v>55.534999999999997</v>
       </c>
-      <c r="S37" s="8">
+      <c r="S37" s="7">
         <v>59.412999999999997</v>
       </c>
     </row>
@@ -1086,43 +1182,43 @@
       <c r="N38" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="O38" s="8">
+      <c r="O38" s="7">
         <v>63.16</v>
       </c>
-      <c r="P38" s="8">
+      <c r="P38" s="7">
         <v>53.555</v>
       </c>
-      <c r="Q38" s="8">
+      <c r="Q38" s="7">
         <v>58.774999999999999</v>
       </c>
-      <c r="R38" s="8">
+      <c r="R38" s="7">
         <v>50.853999999999999</v>
       </c>
-      <c r="S38" s="8">
+      <c r="S38" s="7">
         <v>55.906999999999996</v>
       </c>
     </row>
     <row r="39" spans="14:19" x14ac:dyDescent="0.2">
-      <c r="N39" s="6" t="s">
+      <c r="N39" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="O39" s="7">
+      <c r="O39" s="6">
         <f>AVERAGE(O34:O38)</f>
         <v>60.775999999999996</v>
       </c>
-      <c r="P39" s="7">
+      <c r="P39" s="6">
         <f t="shared" ref="P39" si="9">AVERAGE(P34:P38)</f>
         <v>55.774799999999992</v>
       </c>
-      <c r="Q39" s="7">
+      <c r="Q39" s="6">
         <f t="shared" ref="Q39" si="10">AVERAGE(Q34:Q38)</f>
         <v>53.395600000000002</v>
       </c>
-      <c r="R39" s="7">
+      <c r="R39" s="6">
         <f t="shared" ref="R39" si="11">AVERAGE(R34:R38)</f>
         <v>55.400800000000004</v>
       </c>
-      <c r="S39" s="7">
+      <c r="S39" s="6">
         <f t="shared" ref="S39" si="12">AVERAGE(S34:S38)</f>
         <v>58.275800000000004</v>
       </c>
@@ -1138,4 +1234,1134 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED359FAA-6388-4146-B59F-B62AFCE25D78}">
+  <dimension ref="A1:S39"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A1" s="10"/>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
+      <c r="H1" s="10"/>
+      <c r="I1" s="10"/>
+      <c r="J1" s="10"/>
+      <c r="K1" s="10"/>
+      <c r="L1" s="10"/>
+      <c r="M1" s="10"/>
+      <c r="N1" s="10"/>
+      <c r="O1" s="10"/>
+      <c r="P1" s="10"/>
+      <c r="Q1" s="10"/>
+      <c r="R1" s="10"/>
+      <c r="S1" s="10"/>
+    </row>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A2" s="10"/>
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
+      <c r="G2" s="10"/>
+      <c r="H2" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="I2" s="19"/>
+      <c r="J2" s="19"/>
+      <c r="K2" s="19"/>
+      <c r="L2" s="19"/>
+      <c r="M2" s="19"/>
+      <c r="N2" s="19"/>
+      <c r="O2" s="19"/>
+      <c r="P2" s="19"/>
+      <c r="Q2" s="10"/>
+      <c r="R2" s="10"/>
+      <c r="S2" s="10"/>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A3" s="10"/>
+      <c r="B3" s="10"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="10"/>
+      <c r="G3" s="10"/>
+      <c r="H3" s="19"/>
+      <c r="I3" s="19"/>
+      <c r="J3" s="19"/>
+      <c r="K3" s="19"/>
+      <c r="L3" s="19"/>
+      <c r="M3" s="19"/>
+      <c r="N3" s="19"/>
+      <c r="O3" s="19"/>
+      <c r="P3" s="19"/>
+      <c r="Q3" s="10"/>
+      <c r="R3" s="10"/>
+      <c r="S3" s="10"/>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A4" s="10"/>
+      <c r="B4" s="10"/>
+      <c r="C4" s="10"/>
+      <c r="D4" s="10"/>
+      <c r="E4" s="10"/>
+      <c r="F4" s="10"/>
+      <c r="G4" s="10"/>
+      <c r="H4" s="10"/>
+      <c r="I4" s="10"/>
+      <c r="J4" s="10"/>
+      <c r="K4" s="10"/>
+      <c r="L4" s="10"/>
+      <c r="M4" s="10"/>
+      <c r="N4" s="10"/>
+      <c r="O4" s="10"/>
+      <c r="P4" s="10"/>
+      <c r="Q4" s="10"/>
+      <c r="R4" s="10"/>
+      <c r="S4" s="10"/>
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A5" s="10"/>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="10"/>
+      <c r="F5" s="10"/>
+      <c r="G5" s="10"/>
+      <c r="H5" s="10"/>
+      <c r="I5" s="10"/>
+      <c r="J5" s="10"/>
+      <c r="K5" s="10"/>
+      <c r="L5" s="10"/>
+      <c r="M5" s="10"/>
+      <c r="N5" s="10"/>
+      <c r="O5" s="10"/>
+      <c r="P5" s="10"/>
+      <c r="Q5" s="10"/>
+      <c r="R5" s="10"/>
+      <c r="S5" s="10"/>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A6" s="10"/>
+      <c r="B6" s="10"/>
+      <c r="C6" s="10"/>
+      <c r="D6" s="10"/>
+      <c r="E6" s="20" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" s="20"/>
+      <c r="G6" s="20"/>
+      <c r="H6" s="20"/>
+      <c r="I6" s="20"/>
+      <c r="J6" s="20"/>
+      <c r="K6" s="10"/>
+      <c r="L6" s="10"/>
+      <c r="M6" s="10"/>
+      <c r="N6" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="O6" s="20"/>
+      <c r="P6" s="20"/>
+      <c r="Q6" s="20"/>
+      <c r="R6" s="20"/>
+      <c r="S6" s="20"/>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A7" s="10"/>
+      <c r="B7" s="10"/>
+      <c r="C7" s="10"/>
+      <c r="D7" s="10"/>
+      <c r="E7" s="10"/>
+      <c r="F7" s="10"/>
+      <c r="G7" s="10"/>
+      <c r="H7" s="10"/>
+      <c r="I7" s="10"/>
+      <c r="J7" s="10"/>
+      <c r="K7" s="10"/>
+      <c r="L7" s="10"/>
+      <c r="M7" s="10"/>
+      <c r="N7" s="10"/>
+      <c r="O7" s="10"/>
+      <c r="P7" s="10"/>
+      <c r="Q7" s="10"/>
+      <c r="R7" s="10"/>
+      <c r="S7" s="10"/>
+    </row>
+    <row r="8" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A8" s="10"/>
+      <c r="B8" s="10"/>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="10"/>
+      <c r="F8" s="11">
+        <v>100</v>
+      </c>
+      <c r="G8" s="12">
+        <v>1000</v>
+      </c>
+      <c r="H8" s="12">
+        <v>10000</v>
+      </c>
+      <c r="I8" s="12">
+        <v>100000</v>
+      </c>
+      <c r="J8" s="12">
+        <v>150000</v>
+      </c>
+      <c r="K8" s="10"/>
+      <c r="L8" s="10"/>
+      <c r="M8" s="10"/>
+      <c r="N8" s="10"/>
+      <c r="O8" s="11">
+        <v>100</v>
+      </c>
+      <c r="P8" s="12">
+        <v>1000</v>
+      </c>
+      <c r="Q8" s="12">
+        <v>10000</v>
+      </c>
+      <c r="R8" s="12">
+        <v>100000</v>
+      </c>
+      <c r="S8" s="12">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A9" s="10"/>
+      <c r="B9" s="10"/>
+      <c r="C9" s="10"/>
+      <c r="D9" s="10"/>
+      <c r="E9" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="F9" s="13">
+        <v>33.566000000000003</v>
+      </c>
+      <c r="G9" s="13">
+        <v>34.405999999999999</v>
+      </c>
+      <c r="H9" s="14"/>
+      <c r="I9" s="14"/>
+      <c r="J9" s="14"/>
+      <c r="K9" s="10"/>
+      <c r="L9" s="10"/>
+      <c r="M9" s="10"/>
+      <c r="N9" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="O9" s="15">
+        <v>77.754999999999995</v>
+      </c>
+      <c r="P9" s="15">
+        <v>119.75700000000001</v>
+      </c>
+      <c r="Q9" s="15">
+        <v>165.14099999999999</v>
+      </c>
+      <c r="R9" s="15">
+        <v>229.625</v>
+      </c>
+      <c r="S9" s="15">
+        <v>308.29300000000001</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A10" s="10"/>
+      <c r="B10" s="10"/>
+      <c r="C10" s="10"/>
+      <c r="D10" s="10"/>
+      <c r="E10" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="F10" s="13">
+        <v>31.742000000000001</v>
+      </c>
+      <c r="G10" s="13">
+        <v>38.517000000000003</v>
+      </c>
+      <c r="H10" s="14"/>
+      <c r="I10" s="14"/>
+      <c r="J10" s="14"/>
+      <c r="K10" s="10"/>
+      <c r="L10" s="10"/>
+      <c r="M10" s="10"/>
+      <c r="N10" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="O10" s="15">
+        <v>76.718999999999994</v>
+      </c>
+      <c r="P10" s="15">
+        <v>99.938999999999993</v>
+      </c>
+      <c r="Q10" s="15">
+        <v>190.42500000000001</v>
+      </c>
+      <c r="R10" s="15">
+        <v>239.77799999999999</v>
+      </c>
+      <c r="S10" s="15">
+        <v>275.48099999999999</v>
+      </c>
+    </row>
+    <row r="11" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A11" s="10"/>
+      <c r="B11" s="10"/>
+      <c r="C11" s="10"/>
+      <c r="D11" s="10"/>
+      <c r="E11" s="16" t="s">
+        <v>2</v>
+      </c>
+      <c r="F11" s="13">
+        <v>30.007000000000001</v>
+      </c>
+      <c r="G11" s="13">
+        <v>36.417999999999999</v>
+      </c>
+      <c r="H11" s="14"/>
+      <c r="I11" s="14"/>
+      <c r="J11" s="14"/>
+      <c r="K11" s="10"/>
+      <c r="L11" s="10"/>
+      <c r="M11" s="10"/>
+      <c r="N11" s="16" t="s">
+        <v>2</v>
+      </c>
+      <c r="O11" s="15">
+        <v>140.524</v>
+      </c>
+      <c r="P11" s="15">
+        <v>97.105999999999995</v>
+      </c>
+      <c r="Q11" s="15">
+        <v>208.499</v>
+      </c>
+      <c r="R11" s="15">
+        <v>242.53899999999999</v>
+      </c>
+      <c r="S11" s="15">
+        <v>228.61699999999999</v>
+      </c>
+    </row>
+    <row r="12" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A12" s="10"/>
+      <c r="B12" s="10"/>
+      <c r="C12" s="10"/>
+      <c r="D12" s="10"/>
+      <c r="E12" s="16" t="s">
+        <v>3</v>
+      </c>
+      <c r="F12" s="13">
+        <v>33.454000000000001</v>
+      </c>
+      <c r="G12" s="13"/>
+      <c r="H12" s="14"/>
+      <c r="I12" s="14"/>
+      <c r="J12" s="14"/>
+      <c r="K12" s="10"/>
+      <c r="L12" s="10"/>
+      <c r="M12" s="10"/>
+      <c r="N12" s="16" t="s">
+        <v>3</v>
+      </c>
+      <c r="O12" s="15">
+        <v>97.156000000000006</v>
+      </c>
+      <c r="P12" s="15">
+        <v>99.393000000000001</v>
+      </c>
+      <c r="Q12" s="15">
+        <v>172.39699999999999</v>
+      </c>
+      <c r="R12" s="15">
+        <v>278.01600000000002</v>
+      </c>
+      <c r="S12" s="15">
+        <v>233.97800000000001</v>
+      </c>
+    </row>
+    <row r="13" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A13" s="10"/>
+      <c r="B13" s="10"/>
+      <c r="C13" s="10"/>
+      <c r="D13" s="10"/>
+      <c r="E13" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="F13" s="13">
+        <v>31.077999999999999</v>
+      </c>
+      <c r="G13" s="13"/>
+      <c r="H13" s="14"/>
+      <c r="I13" s="14"/>
+      <c r="J13" s="14"/>
+      <c r="K13" s="10"/>
+      <c r="L13" s="10"/>
+      <c r="M13" s="10"/>
+      <c r="N13" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="O13" s="15">
+        <v>77.403000000000006</v>
+      </c>
+      <c r="P13" s="15">
+        <v>103.63500000000001</v>
+      </c>
+      <c r="Q13" s="15">
+        <v>159.054</v>
+      </c>
+      <c r="R13" s="15">
+        <v>240.28299999999999</v>
+      </c>
+      <c r="S13" s="15">
+        <v>249.54400000000001</v>
+      </c>
+    </row>
+    <row r="14" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A14" s="10"/>
+      <c r="B14" s="10"/>
+      <c r="C14" s="10"/>
+      <c r="D14" s="10"/>
+      <c r="E14" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="F14" s="18"/>
+      <c r="G14" s="18"/>
+      <c r="H14" s="18"/>
+      <c r="I14" s="18"/>
+      <c r="J14" s="18"/>
+      <c r="K14" s="10"/>
+      <c r="L14" s="10"/>
+      <c r="M14" s="10"/>
+      <c r="N14" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="O14" s="18">
+        <v>93.911000000000001</v>
+      </c>
+      <c r="P14" s="18">
+        <v>103.96599999999999</v>
+      </c>
+      <c r="Q14" s="18">
+        <v>179.10300000000001</v>
+      </c>
+      <c r="R14" s="18">
+        <v>246.048</v>
+      </c>
+      <c r="S14" s="18">
+        <v>259.18299999999999</v>
+      </c>
+    </row>
+    <row r="15" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A15" s="10"/>
+      <c r="B15" s="10"/>
+      <c r="C15" s="10"/>
+      <c r="D15" s="10"/>
+      <c r="E15" s="10"/>
+      <c r="F15" s="10"/>
+      <c r="G15" s="10"/>
+      <c r="H15" s="10"/>
+      <c r="I15" s="10"/>
+      <c r="J15" s="10"/>
+      <c r="K15" s="10"/>
+      <c r="L15" s="10"/>
+      <c r="M15" s="10"/>
+      <c r="N15" s="10"/>
+      <c r="O15" s="10"/>
+      <c r="P15" s="10"/>
+      <c r="Q15" s="10"/>
+      <c r="R15" s="10"/>
+      <c r="S15" s="10"/>
+    </row>
+    <row r="16" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A16" s="10"/>
+      <c r="B16" s="10"/>
+      <c r="C16" s="10"/>
+      <c r="D16" s="10"/>
+      <c r="E16" s="10"/>
+      <c r="F16" s="10"/>
+      <c r="G16" s="10"/>
+      <c r="H16" s="10"/>
+      <c r="I16" s="10"/>
+      <c r="J16" s="10"/>
+      <c r="K16" s="10"/>
+      <c r="L16" s="10"/>
+      <c r="M16" s="10"/>
+      <c r="N16" s="10"/>
+      <c r="O16" s="10"/>
+      <c r="P16" s="10"/>
+      <c r="Q16" s="10"/>
+      <c r="R16" s="10"/>
+      <c r="S16" s="10"/>
+    </row>
+    <row r="17" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A17" s="10"/>
+      <c r="B17" s="10"/>
+      <c r="C17" s="10"/>
+      <c r="D17" s="10"/>
+      <c r="E17" s="10"/>
+      <c r="F17" s="10"/>
+      <c r="G17" s="10"/>
+      <c r="H17" s="10"/>
+      <c r="I17" s="10"/>
+      <c r="J17" s="10"/>
+      <c r="K17" s="10"/>
+      <c r="L17" s="10"/>
+      <c r="M17" s="10"/>
+      <c r="N17" s="10"/>
+      <c r="O17" s="10"/>
+      <c r="P17" s="10"/>
+      <c r="Q17" s="10"/>
+      <c r="R17" s="10"/>
+      <c r="S17" s="10"/>
+    </row>
+    <row r="18" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A18" s="10"/>
+      <c r="B18" s="10"/>
+      <c r="C18" s="10"/>
+      <c r="D18" s="10"/>
+      <c r="E18" s="10"/>
+      <c r="F18" s="10"/>
+      <c r="G18" s="10"/>
+      <c r="H18" s="10"/>
+      <c r="I18" s="10"/>
+      <c r="J18" s="10"/>
+      <c r="K18" s="10"/>
+      <c r="L18" s="10"/>
+      <c r="M18" s="10"/>
+      <c r="N18" s="10"/>
+      <c r="O18" s="10"/>
+      <c r="P18" s="10"/>
+      <c r="Q18" s="10"/>
+      <c r="R18" s="10"/>
+      <c r="S18" s="10"/>
+    </row>
+    <row r="19" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A19" s="10"/>
+      <c r="B19" s="10"/>
+      <c r="C19" s="10"/>
+      <c r="D19" s="10"/>
+      <c r="E19" s="10"/>
+      <c r="F19" s="10"/>
+      <c r="G19" s="10"/>
+      <c r="H19" s="10"/>
+      <c r="I19" s="10"/>
+      <c r="J19" s="10"/>
+      <c r="K19" s="10"/>
+      <c r="L19" s="10"/>
+      <c r="M19" s="10"/>
+      <c r="N19" s="10"/>
+      <c r="O19" s="10"/>
+      <c r="P19" s="10"/>
+      <c r="Q19" s="10"/>
+      <c r="R19" s="10"/>
+      <c r="S19" s="10"/>
+    </row>
+    <row r="20" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A20" s="10"/>
+      <c r="B20" s="10"/>
+      <c r="C20" s="10"/>
+      <c r="D20" s="10"/>
+      <c r="E20" s="10"/>
+      <c r="F20" s="10"/>
+      <c r="G20" s="10"/>
+      <c r="H20" s="10"/>
+      <c r="I20" s="10"/>
+      <c r="J20" s="10"/>
+      <c r="K20" s="10"/>
+      <c r="L20" s="10"/>
+      <c r="M20" s="10"/>
+      <c r="N20" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="O20" s="20"/>
+      <c r="P20" s="20"/>
+      <c r="Q20" s="20"/>
+      <c r="R20" s="20"/>
+      <c r="S20" s="20"/>
+    </row>
+    <row r="21" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A21" s="10"/>
+      <c r="B21" s="10"/>
+      <c r="C21" s="10"/>
+      <c r="D21" s="10"/>
+      <c r="E21" s="10"/>
+      <c r="F21" s="10"/>
+      <c r="G21" s="10"/>
+      <c r="H21" s="10"/>
+      <c r="I21" s="10"/>
+      <c r="J21" s="10"/>
+      <c r="K21" s="10"/>
+      <c r="L21" s="10"/>
+      <c r="M21" s="10"/>
+      <c r="N21" s="10"/>
+      <c r="O21" s="10"/>
+      <c r="P21" s="10"/>
+      <c r="Q21" s="10"/>
+      <c r="R21" s="10"/>
+      <c r="S21" s="10"/>
+    </row>
+    <row r="22" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A22" s="10"/>
+      <c r="B22" s="10"/>
+      <c r="C22" s="10"/>
+      <c r="D22" s="10"/>
+      <c r="E22" s="10"/>
+      <c r="F22" s="10"/>
+      <c r="G22" s="10"/>
+      <c r="H22" s="10"/>
+      <c r="I22" s="10"/>
+      <c r="J22" s="10"/>
+      <c r="K22" s="10"/>
+      <c r="L22" s="10"/>
+      <c r="M22" s="10"/>
+      <c r="N22" s="10"/>
+      <c r="O22" s="11">
+        <v>100</v>
+      </c>
+      <c r="P22" s="12">
+        <v>1000</v>
+      </c>
+      <c r="Q22" s="12">
+        <v>10000</v>
+      </c>
+      <c r="R22" s="12">
+        <v>100000</v>
+      </c>
+      <c r="S22" s="12">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="23" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A23" s="10"/>
+      <c r="B23" s="10"/>
+      <c r="C23" s="10"/>
+      <c r="D23" s="10"/>
+      <c r="E23" s="10"/>
+      <c r="F23" s="10"/>
+      <c r="G23" s="10"/>
+      <c r="H23" s="10"/>
+      <c r="I23" s="10"/>
+      <c r="J23" s="10"/>
+      <c r="K23" s="10"/>
+      <c r="L23" s="10"/>
+      <c r="M23" s="10"/>
+      <c r="N23" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="O23" s="15">
+        <v>75.866</v>
+      </c>
+      <c r="P23" s="15">
+        <v>130.58199999999999</v>
+      </c>
+      <c r="Q23" s="15">
+        <v>152.541</v>
+      </c>
+      <c r="R23" s="15">
+        <v>249.38900000000001</v>
+      </c>
+      <c r="S23" s="15">
+        <v>232.51900000000001</v>
+      </c>
+    </row>
+    <row r="24" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A24" s="10"/>
+      <c r="B24" s="10"/>
+      <c r="C24" s="10"/>
+      <c r="D24" s="10"/>
+      <c r="E24" s="10"/>
+      <c r="F24" s="10"/>
+      <c r="G24" s="10"/>
+      <c r="H24" s="10"/>
+      <c r="I24" s="10"/>
+      <c r="J24" s="10"/>
+      <c r="K24" s="10"/>
+      <c r="L24" s="10"/>
+      <c r="M24" s="10"/>
+      <c r="N24" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="O24" s="15">
+        <v>94.698999999999998</v>
+      </c>
+      <c r="P24" s="15">
+        <v>99.510999999999996</v>
+      </c>
+      <c r="Q24" s="15">
+        <v>184.23699999999999</v>
+      </c>
+      <c r="R24" s="15">
+        <v>255.25399999999999</v>
+      </c>
+      <c r="S24" s="15">
+        <v>265.57600000000002</v>
+      </c>
+    </row>
+    <row r="25" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A25" s="10"/>
+      <c r="B25" s="10"/>
+      <c r="C25" s="10"/>
+      <c r="D25" s="10"/>
+      <c r="E25" s="10"/>
+      <c r="F25" s="10"/>
+      <c r="G25" s="10"/>
+      <c r="H25" s="10"/>
+      <c r="I25" s="10"/>
+      <c r="J25" s="10"/>
+      <c r="K25" s="10"/>
+      <c r="L25" s="10"/>
+      <c r="M25" s="10"/>
+      <c r="N25" s="16" t="s">
+        <v>2</v>
+      </c>
+      <c r="O25" s="15">
+        <v>102.77</v>
+      </c>
+      <c r="P25" s="15">
+        <v>100.2</v>
+      </c>
+      <c r="Q25" s="15">
+        <v>175.64099999999999</v>
+      </c>
+      <c r="R25" s="15">
+        <v>230.971</v>
+      </c>
+      <c r="S25" s="15">
+        <v>270.988</v>
+      </c>
+    </row>
+    <row r="26" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A26" s="10"/>
+      <c r="B26" s="10"/>
+      <c r="C26" s="10"/>
+      <c r="D26" s="10"/>
+      <c r="E26" s="10"/>
+      <c r="F26" s="10"/>
+      <c r="G26" s="10"/>
+      <c r="H26" s="10"/>
+      <c r="I26" s="10"/>
+      <c r="J26" s="10"/>
+      <c r="K26" s="10"/>
+      <c r="L26" s="10"/>
+      <c r="M26" s="10"/>
+      <c r="N26" s="16" t="s">
+        <v>3</v>
+      </c>
+      <c r="O26" s="15">
+        <v>78.587000000000003</v>
+      </c>
+      <c r="P26" s="15">
+        <v>114.334</v>
+      </c>
+      <c r="Q26" s="15">
+        <v>210.39599999999999</v>
+      </c>
+      <c r="R26" s="15">
+        <v>261.68400000000003</v>
+      </c>
+      <c r="S26" s="15">
+        <v>242.14</v>
+      </c>
+    </row>
+    <row r="27" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A27" s="10"/>
+      <c r="B27" s="10"/>
+      <c r="C27" s="10"/>
+      <c r="D27" s="10"/>
+      <c r="E27" s="10"/>
+      <c r="F27" s="10"/>
+      <c r="G27" s="10"/>
+      <c r="H27" s="10"/>
+      <c r="I27" s="10"/>
+      <c r="J27" s="10"/>
+      <c r="K27" s="10"/>
+      <c r="L27" s="10"/>
+      <c r="M27" s="10"/>
+      <c r="N27" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="O27" s="15">
+        <v>87.555000000000007</v>
+      </c>
+      <c r="P27" s="15">
+        <v>110.733</v>
+      </c>
+      <c r="Q27" s="15">
+        <v>160.60300000000001</v>
+      </c>
+      <c r="R27" s="15">
+        <v>240.37</v>
+      </c>
+      <c r="S27" s="15">
+        <v>245.50899999999999</v>
+      </c>
+    </row>
+    <row r="28" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A28" s="10"/>
+      <c r="B28" s="10"/>
+      <c r="C28" s="10"/>
+      <c r="D28" s="10"/>
+      <c r="E28" s="10"/>
+      <c r="F28" s="10"/>
+      <c r="G28" s="10"/>
+      <c r="H28" s="10"/>
+      <c r="I28" s="10"/>
+      <c r="J28" s="10"/>
+      <c r="K28" s="10"/>
+      <c r="L28" s="10"/>
+      <c r="M28" s="10"/>
+      <c r="N28" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="O28" s="18">
+        <v>87.894999999999996</v>
+      </c>
+      <c r="P28" s="18">
+        <v>111.072</v>
+      </c>
+      <c r="Q28" s="18">
+        <v>176.684</v>
+      </c>
+      <c r="R28" s="18">
+        <v>247.53399999999999</v>
+      </c>
+      <c r="S28" s="18">
+        <v>251.346</v>
+      </c>
+    </row>
+    <row r="29" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A29" s="10"/>
+      <c r="B29" s="10"/>
+      <c r="C29" s="10"/>
+      <c r="D29" s="10"/>
+      <c r="E29" s="10"/>
+      <c r="F29" s="10"/>
+      <c r="G29" s="10"/>
+      <c r="H29" s="10"/>
+      <c r="I29" s="10"/>
+      <c r="J29" s="10"/>
+      <c r="K29" s="10"/>
+      <c r="L29" s="10"/>
+      <c r="M29" s="10"/>
+      <c r="N29" s="10"/>
+      <c r="O29" s="10"/>
+      <c r="P29" s="10"/>
+      <c r="Q29" s="10"/>
+      <c r="R29" s="10"/>
+      <c r="S29" s="10"/>
+    </row>
+    <row r="30" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A30" s="10"/>
+      <c r="B30" s="10"/>
+      <c r="C30" s="10"/>
+      <c r="D30" s="10"/>
+      <c r="E30" s="10"/>
+      <c r="F30" s="10"/>
+      <c r="G30" s="10"/>
+      <c r="H30" s="10"/>
+      <c r="I30" s="10"/>
+      <c r="J30" s="10"/>
+      <c r="K30" s="10"/>
+      <c r="L30" s="10"/>
+      <c r="M30" s="10"/>
+      <c r="N30" s="10"/>
+      <c r="O30" s="10"/>
+      <c r="P30" s="10"/>
+      <c r="Q30" s="10"/>
+      <c r="R30" s="10"/>
+      <c r="S30" s="10"/>
+    </row>
+    <row r="31" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A31" s="10"/>
+      <c r="B31" s="10"/>
+      <c r="C31" s="10"/>
+      <c r="D31" s="10"/>
+      <c r="E31" s="10"/>
+      <c r="F31" s="10"/>
+      <c r="G31" s="10"/>
+      <c r="H31" s="10"/>
+      <c r="I31" s="10"/>
+      <c r="J31" s="10"/>
+      <c r="K31" s="10"/>
+      <c r="L31" s="10"/>
+      <c r="M31" s="10"/>
+      <c r="N31" s="20" t="s">
+        <v>14</v>
+      </c>
+      <c r="O31" s="20"/>
+      <c r="P31" s="20"/>
+      <c r="Q31" s="20"/>
+      <c r="R31" s="20"/>
+      <c r="S31" s="20"/>
+    </row>
+    <row r="32" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A32" s="10"/>
+      <c r="B32" s="10"/>
+      <c r="C32" s="10"/>
+      <c r="D32" s="10"/>
+      <c r="E32" s="10"/>
+      <c r="F32" s="10"/>
+      <c r="G32" s="10"/>
+      <c r="H32" s="10"/>
+      <c r="I32" s="10"/>
+      <c r="J32" s="10"/>
+      <c r="K32" s="10"/>
+      <c r="L32" s="10"/>
+      <c r="M32" s="10"/>
+      <c r="N32" s="10"/>
+      <c r="O32" s="10"/>
+      <c r="P32" s="10"/>
+      <c r="Q32" s="10"/>
+      <c r="R32" s="10"/>
+      <c r="S32" s="10"/>
+    </row>
+    <row r="33" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A33" s="10"/>
+      <c r="B33" s="10"/>
+      <c r="C33" s="10"/>
+      <c r="D33" s="10"/>
+      <c r="E33" s="10"/>
+      <c r="F33" s="10"/>
+      <c r="G33" s="10"/>
+      <c r="H33" s="10"/>
+      <c r="I33" s="10"/>
+      <c r="J33" s="10"/>
+      <c r="K33" s="10"/>
+      <c r="L33" s="10"/>
+      <c r="M33" s="10"/>
+      <c r="N33" s="10"/>
+      <c r="O33" s="11">
+        <v>100</v>
+      </c>
+      <c r="P33" s="12">
+        <v>1000</v>
+      </c>
+      <c r="Q33" s="12">
+        <v>10000</v>
+      </c>
+      <c r="R33" s="12">
+        <v>100000</v>
+      </c>
+      <c r="S33" s="12">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="34" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A34" s="10"/>
+      <c r="B34" s="10"/>
+      <c r="C34" s="10"/>
+      <c r="D34" s="10"/>
+      <c r="E34" s="10"/>
+      <c r="F34" s="10"/>
+      <c r="G34" s="10"/>
+      <c r="H34" s="10"/>
+      <c r="I34" s="10"/>
+      <c r="J34" s="10"/>
+      <c r="K34" s="10"/>
+      <c r="L34" s="10"/>
+      <c r="M34" s="10"/>
+      <c r="N34" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="O34" s="15">
+        <v>55.804000000000002</v>
+      </c>
+      <c r="P34" s="15">
+        <v>50.383000000000003</v>
+      </c>
+      <c r="Q34" s="15">
+        <v>51.292999999999999</v>
+      </c>
+      <c r="R34" s="15">
+        <v>52.933999999999997</v>
+      </c>
+      <c r="S34" s="15">
+        <v>52.692999999999998</v>
+      </c>
+    </row>
+    <row r="35" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A35" s="10"/>
+      <c r="B35" s="10"/>
+      <c r="C35" s="10"/>
+      <c r="D35" s="10"/>
+      <c r="E35" s="10"/>
+      <c r="F35" s="10"/>
+      <c r="G35" s="10"/>
+      <c r="H35" s="10"/>
+      <c r="I35" s="10"/>
+      <c r="J35" s="10"/>
+      <c r="K35" s="10"/>
+      <c r="L35" s="10"/>
+      <c r="M35" s="10"/>
+      <c r="N35" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="O35" s="15">
+        <v>65.367999999999995</v>
+      </c>
+      <c r="P35" s="15">
+        <v>69.436999999999998</v>
+      </c>
+      <c r="Q35" s="15">
+        <v>51.094999999999999</v>
+      </c>
+      <c r="R35" s="15">
+        <v>52.177</v>
+      </c>
+      <c r="S35" s="15">
+        <v>58.481000000000002</v>
+      </c>
+    </row>
+    <row r="36" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A36" s="10"/>
+      <c r="B36" s="10"/>
+      <c r="C36" s="10"/>
+      <c r="D36" s="10"/>
+      <c r="E36" s="10"/>
+      <c r="F36" s="10"/>
+      <c r="G36" s="10"/>
+      <c r="H36" s="10"/>
+      <c r="I36" s="10"/>
+      <c r="J36" s="10"/>
+      <c r="K36" s="10"/>
+      <c r="L36" s="10"/>
+      <c r="M36" s="10"/>
+      <c r="N36" s="16" t="s">
+        <v>2</v>
+      </c>
+      <c r="O36" s="15">
+        <v>56.311</v>
+      </c>
+      <c r="P36" s="15">
+        <v>53.951999999999998</v>
+      </c>
+      <c r="Q36" s="15">
+        <v>52.320999999999998</v>
+      </c>
+      <c r="R36" s="15">
+        <v>65.504000000000005</v>
+      </c>
+      <c r="S36" s="15">
+        <v>64.885000000000005</v>
+      </c>
+    </row>
+    <row r="37" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A37" s="10"/>
+      <c r="B37" s="10"/>
+      <c r="C37" s="10"/>
+      <c r="D37" s="10"/>
+      <c r="E37" s="10"/>
+      <c r="F37" s="10"/>
+      <c r="G37" s="10"/>
+      <c r="H37" s="10"/>
+      <c r="I37" s="10"/>
+      <c r="J37" s="10"/>
+      <c r="K37" s="10"/>
+      <c r="L37" s="10"/>
+      <c r="M37" s="10"/>
+      <c r="N37" s="16" t="s">
+        <v>3</v>
+      </c>
+      <c r="O37" s="15">
+        <v>63.237000000000002</v>
+      </c>
+      <c r="P37" s="15">
+        <v>51.546999999999997</v>
+      </c>
+      <c r="Q37" s="15">
+        <v>53.494</v>
+      </c>
+      <c r="R37" s="15">
+        <v>55.534999999999997</v>
+      </c>
+      <c r="S37" s="15">
+        <v>59.412999999999997</v>
+      </c>
+    </row>
+    <row r="38" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A38" s="10"/>
+      <c r="B38" s="10"/>
+      <c r="C38" s="10"/>
+      <c r="D38" s="10"/>
+      <c r="E38" s="10"/>
+      <c r="F38" s="10"/>
+      <c r="G38" s="10"/>
+      <c r="H38" s="10"/>
+      <c r="I38" s="10"/>
+      <c r="J38" s="10"/>
+      <c r="K38" s="10"/>
+      <c r="L38" s="10"/>
+      <c r="M38" s="10"/>
+      <c r="N38" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="O38" s="15">
+        <v>63.16</v>
+      </c>
+      <c r="P38" s="15">
+        <v>53.555</v>
+      </c>
+      <c r="Q38" s="15">
+        <v>58.774999999999999</v>
+      </c>
+      <c r="R38" s="15">
+        <v>50.853999999999999</v>
+      </c>
+      <c r="S38" s="15">
+        <v>55.906999999999996</v>
+      </c>
+    </row>
+    <row r="39" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A39" s="10"/>
+      <c r="B39" s="10"/>
+      <c r="C39" s="10"/>
+      <c r="D39" s="10"/>
+      <c r="E39" s="10"/>
+      <c r="F39" s="10"/>
+      <c r="G39" s="10"/>
+      <c r="H39" s="10"/>
+      <c r="I39" s="10"/>
+      <c r="J39" s="10"/>
+      <c r="K39" s="10"/>
+      <c r="L39" s="10"/>
+      <c r="M39" s="10"/>
+      <c r="N39" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="O39" s="18">
+        <v>60.776000000000003</v>
+      </c>
+      <c r="P39" s="18">
+        <v>55.774999999999999</v>
+      </c>
+      <c r="Q39" s="18">
+        <v>53.396000000000001</v>
+      </c>
+      <c r="R39" s="18">
+        <v>55.401000000000003</v>
+      </c>
+      <c r="S39" s="18">
+        <v>58.276000000000003</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="H2:P3"/>
+    <mergeCell ref="E6:J6"/>
+    <mergeCell ref="N6:S6"/>
+    <mergeCell ref="N20:S20"/>
+    <mergeCell ref="N31:S31"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add snowflake impl and result snowflake
</commit_message>
<xml_diff>
--- a/docs/result.xlsx
+++ b/docs/result.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/muhammadrayandika/projects/bmkg_weather_forecasting/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C768A098-3E72-9E46-9ED4-66E582A02DFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1862B357-5334-CC49-8664-8AE7585F189B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="700" windowWidth="33600" windowHeight="20280" activeTab="1" xr2:uid="{5AC5918A-7EFC-C743-9AF6-45D314C9895F}"/>
+    <workbookView xWindow="0" yWindow="700" windowWidth="33600" windowHeight="20300" activeTab="1" xr2:uid="{5AC5918A-7EFC-C743-9AF6-45D314C9895F}"/>
   </bookViews>
   <sheets>
     <sheet name="Result Starflake" sheetId="1" r:id="rId1"/>
@@ -166,7 +166,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -226,12 +226,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -248,12 +257,6 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -269,11 +272,23 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="3" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -608,46 +623,46 @@
   </cols>
   <sheetData>
     <row r="2" spans="5:19" x14ac:dyDescent="0.2">
-      <c r="H2" s="9" t="s">
+      <c r="H2" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="I2" s="9"/>
-      <c r="J2" s="9"/>
-      <c r="K2" s="9"/>
-      <c r="L2" s="9"/>
-      <c r="M2" s="9"/>
-      <c r="N2" s="9"/>
-      <c r="O2" s="9"/>
-      <c r="P2" s="9"/>
+      <c r="I2" s="18"/>
+      <c r="J2" s="18"/>
+      <c r="K2" s="18"/>
+      <c r="L2" s="18"/>
+      <c r="M2" s="18"/>
+      <c r="N2" s="18"/>
+      <c r="O2" s="18"/>
+      <c r="P2" s="18"/>
     </row>
     <row r="3" spans="5:19" x14ac:dyDescent="0.2">
-      <c r="H3" s="9"/>
-      <c r="I3" s="9"/>
-      <c r="J3" s="9"/>
-      <c r="K3" s="9"/>
-      <c r="L3" s="9"/>
-      <c r="M3" s="9"/>
-      <c r="N3" s="9"/>
-      <c r="O3" s="9"/>
-      <c r="P3" s="9"/>
+      <c r="H3" s="18"/>
+      <c r="I3" s="18"/>
+      <c r="J3" s="18"/>
+      <c r="K3" s="18"/>
+      <c r="L3" s="18"/>
+      <c r="M3" s="18"/>
+      <c r="N3" s="18"/>
+      <c r="O3" s="18"/>
+      <c r="P3" s="18"/>
     </row>
     <row r="6" spans="5:19" x14ac:dyDescent="0.2">
-      <c r="E6" s="8" t="s">
+      <c r="E6" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="F6" s="8"/>
-      <c r="G6" s="8"/>
-      <c r="H6" s="8"/>
-      <c r="I6" s="8"/>
-      <c r="J6" s="8"/>
-      <c r="N6" s="8" t="s">
+      <c r="F6" s="17"/>
+      <c r="G6" s="17"/>
+      <c r="H6" s="17"/>
+      <c r="I6" s="17"/>
+      <c r="J6" s="17"/>
+      <c r="N6" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="O6" s="8"/>
-      <c r="P6" s="8"/>
-      <c r="Q6" s="8"/>
-      <c r="R6" s="8"/>
-      <c r="S6" s="8"/>
+      <c r="O6" s="17"/>
+      <c r="P6" s="17"/>
+      <c r="Q6" s="17"/>
+      <c r="R6" s="17"/>
+      <c r="S6" s="17"/>
     </row>
     <row r="8" spans="5:19" x14ac:dyDescent="0.2">
       <c r="F8" s="2">
@@ -920,14 +935,14 @@
       </c>
     </row>
     <row r="20" spans="14:19" x14ac:dyDescent="0.2">
-      <c r="N20" s="8" t="s">
+      <c r="N20" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="O20" s="8"/>
-      <c r="P20" s="8"/>
-      <c r="Q20" s="8"/>
-      <c r="R20" s="8"/>
-      <c r="S20" s="8"/>
+      <c r="O20" s="17"/>
+      <c r="P20" s="17"/>
+      <c r="Q20" s="17"/>
+      <c r="R20" s="17"/>
+      <c r="S20" s="17"/>
     </row>
     <row r="22" spans="14:19" x14ac:dyDescent="0.2">
       <c r="O22" s="2">
@@ -1072,14 +1087,14 @@
       </c>
     </row>
     <row r="31" spans="14:19" x14ac:dyDescent="0.2">
-      <c r="N31" s="8" t="s">
+      <c r="N31" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="O31" s="8"/>
-      <c r="P31" s="8"/>
-      <c r="Q31" s="8"/>
-      <c r="R31" s="8"/>
-      <c r="S31" s="8"/>
+      <c r="O31" s="17"/>
+      <c r="P31" s="17"/>
+      <c r="Q31" s="17"/>
+      <c r="R31" s="17"/>
+      <c r="S31" s="17"/>
     </row>
     <row r="33" spans="14:19" x14ac:dyDescent="0.2">
       <c r="O33" s="2">
@@ -1242,34 +1257,34 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A1" s="10"/>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
-      <c r="H1" s="10"/>
-      <c r="I1" s="10"/>
-      <c r="J1" s="10"/>
-      <c r="K1" s="10"/>
-      <c r="L1" s="10"/>
-      <c r="M1" s="10"/>
-      <c r="N1" s="10"/>
-      <c r="O1" s="10"/>
-      <c r="P1" s="10"/>
-      <c r="Q1" s="10"/>
-      <c r="R1" s="10"/>
-      <c r="S1" s="10"/>
+      <c r="A1" s="8"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+      <c r="H1" s="8"/>
+      <c r="I1" s="8"/>
+      <c r="J1" s="8"/>
+      <c r="K1" s="8"/>
+      <c r="L1" s="8"/>
+      <c r="M1" s="8"/>
+      <c r="N1" s="8"/>
+      <c r="O1" s="8"/>
+      <c r="P1" s="8"/>
+      <c r="Q1" s="8"/>
+      <c r="R1" s="8"/>
+      <c r="S1" s="8"/>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A2" s="10"/>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
-      <c r="G2" s="10"/>
+      <c r="A2" s="8"/>
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
       <c r="H2" s="19" t="s">
         <v>10</v>
       </c>
@@ -1281,18 +1296,18 @@
       <c r="N2" s="19"/>
       <c r="O2" s="19"/>
       <c r="P2" s="19"/>
-      <c r="Q2" s="10"/>
-      <c r="R2" s="10"/>
-      <c r="S2" s="10"/>
+      <c r="Q2" s="8"/>
+      <c r="R2" s="8"/>
+      <c r="S2" s="8"/>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A3" s="10"/>
-      <c r="B3" s="10"/>
-      <c r="C3" s="10"/>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10"/>
-      <c r="G3" s="10"/>
+      <c r="A3" s="8"/>
+      <c r="B3" s="8"/>
+      <c r="C3" s="8"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="8"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="8"/>
       <c r="H3" s="19"/>
       <c r="I3" s="19"/>
       <c r="J3" s="19"/>
@@ -1302,57 +1317,57 @@
       <c r="N3" s="19"/>
       <c r="O3" s="19"/>
       <c r="P3" s="19"/>
-      <c r="Q3" s="10"/>
-      <c r="R3" s="10"/>
-      <c r="S3" s="10"/>
+      <c r="Q3" s="8"/>
+      <c r="R3" s="8"/>
+      <c r="S3" s="8"/>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A4" s="10"/>
-      <c r="B4" s="10"/>
-      <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
-      <c r="E4" s="10"/>
-      <c r="F4" s="10"/>
-      <c r="G4" s="10"/>
-      <c r="H4" s="10"/>
-      <c r="I4" s="10"/>
-      <c r="J4" s="10"/>
-      <c r="K4" s="10"/>
-      <c r="L4" s="10"/>
-      <c r="M4" s="10"/>
-      <c r="N4" s="10"/>
-      <c r="O4" s="10"/>
-      <c r="P4" s="10"/>
-      <c r="Q4" s="10"/>
-      <c r="R4" s="10"/>
-      <c r="S4" s="10"/>
+      <c r="A4" s="8"/>
+      <c r="B4" s="8"/>
+      <c r="C4" s="8"/>
+      <c r="D4" s="8"/>
+      <c r="E4" s="8"/>
+      <c r="F4" s="8"/>
+      <c r="G4" s="8"/>
+      <c r="H4" s="8"/>
+      <c r="I4" s="8"/>
+      <c r="J4" s="8"/>
+      <c r="K4" s="8"/>
+      <c r="L4" s="8"/>
+      <c r="M4" s="8"/>
+      <c r="N4" s="8"/>
+      <c r="O4" s="8"/>
+      <c r="P4" s="8"/>
+      <c r="Q4" s="8"/>
+      <c r="R4" s="8"/>
+      <c r="S4" s="8"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A5" s="10"/>
-      <c r="B5" s="10"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="10"/>
-      <c r="F5" s="10"/>
-      <c r="G5" s="10"/>
-      <c r="H5" s="10"/>
-      <c r="I5" s="10"/>
-      <c r="J5" s="10"/>
-      <c r="K5" s="10"/>
-      <c r="L5" s="10"/>
-      <c r="M5" s="10"/>
-      <c r="N5" s="10"/>
-      <c r="O5" s="10"/>
-      <c r="P5" s="10"/>
-      <c r="Q5" s="10"/>
-      <c r="R5" s="10"/>
-      <c r="S5" s="10"/>
+      <c r="A5" s="8"/>
+      <c r="B5" s="8"/>
+      <c r="C5" s="8"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="8"/>
+      <c r="F5" s="8"/>
+      <c r="G5" s="8"/>
+      <c r="H5" s="8"/>
+      <c r="I5" s="8"/>
+      <c r="J5" s="8"/>
+      <c r="K5" s="8"/>
+      <c r="L5" s="8"/>
+      <c r="M5" s="8"/>
+      <c r="N5" s="8"/>
+      <c r="O5" s="8"/>
+      <c r="P5" s="8"/>
+      <c r="Q5" s="8"/>
+      <c r="R5" s="8"/>
+      <c r="S5" s="8"/>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A6" s="10"/>
-      <c r="B6" s="10"/>
-      <c r="C6" s="10"/>
-      <c r="D6" s="10"/>
+      <c r="A6" s="8"/>
+      <c r="B6" s="8"/>
+      <c r="C6" s="8"/>
+      <c r="D6" s="8"/>
       <c r="E6" s="20" t="s">
         <v>11</v>
       </c>
@@ -1361,9 +1376,9 @@
       <c r="H6" s="20"/>
       <c r="I6" s="20"/>
       <c r="J6" s="20"/>
-      <c r="K6" s="10"/>
-      <c r="L6" s="10"/>
-      <c r="M6" s="10"/>
+      <c r="K6" s="8"/>
+      <c r="L6" s="8"/>
+      <c r="M6" s="8"/>
       <c r="N6" s="20" t="s">
         <v>12</v>
       </c>
@@ -1374,412 +1389,466 @@
       <c r="S6" s="20"/>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A7" s="10"/>
-      <c r="B7" s="10"/>
-      <c r="C7" s="10"/>
-      <c r="D7" s="10"/>
-      <c r="E7" s="10"/>
-      <c r="F7" s="10"/>
-      <c r="G7" s="10"/>
-      <c r="H7" s="10"/>
-      <c r="I7" s="10"/>
-      <c r="J7" s="10"/>
-      <c r="K7" s="10"/>
-      <c r="L7" s="10"/>
-      <c r="M7" s="10"/>
-      <c r="N7" s="10"/>
-      <c r="O7" s="10"/>
-      <c r="P7" s="10"/>
-      <c r="Q7" s="10"/>
-      <c r="R7" s="10"/>
-      <c r="S7" s="10"/>
+      <c r="A7" s="8"/>
+      <c r="B7" s="8"/>
+      <c r="C7" s="8"/>
+      <c r="D7" s="8"/>
+      <c r="E7" s="8"/>
+      <c r="F7" s="8"/>
+      <c r="G7" s="8"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="8"/>
+      <c r="J7" s="8"/>
+      <c r="K7" s="8"/>
+      <c r="L7" s="8"/>
+      <c r="M7" s="8"/>
+      <c r="N7" s="8"/>
+      <c r="O7" s="8"/>
+      <c r="P7" s="8"/>
+      <c r="Q7" s="8"/>
+      <c r="R7" s="8"/>
+      <c r="S7" s="8"/>
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A8" s="10"/>
-      <c r="B8" s="10"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="10"/>
-      <c r="F8" s="11">
+      <c r="A8" s="8"/>
+      <c r="B8" s="8"/>
+      <c r="C8" s="8"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="9">
         <v>100</v>
       </c>
-      <c r="G8" s="12">
+      <c r="G8" s="10">
         <v>1000</v>
       </c>
-      <c r="H8" s="12">
+      <c r="H8" s="10">
         <v>10000</v>
       </c>
-      <c r="I8" s="12">
+      <c r="I8" s="10">
         <v>100000</v>
       </c>
-      <c r="J8" s="12">
+      <c r="J8" s="10">
         <v>150000</v>
       </c>
-      <c r="K8" s="10"/>
-      <c r="L8" s="10"/>
-      <c r="M8" s="10"/>
-      <c r="N8" s="10"/>
-      <c r="O8" s="11">
+      <c r="K8" s="8"/>
+      <c r="L8" s="8"/>
+      <c r="M8" s="8"/>
+      <c r="N8" s="8"/>
+      <c r="O8" s="9">
         <v>100</v>
       </c>
-      <c r="P8" s="12">
+      <c r="P8" s="10">
         <v>1000</v>
       </c>
-      <c r="Q8" s="12">
+      <c r="Q8" s="10">
         <v>10000</v>
       </c>
-      <c r="R8" s="12">
+      <c r="R8" s="10">
         <v>100000</v>
       </c>
-      <c r="S8" s="12">
+      <c r="S8" s="10">
         <v>150000</v>
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A9" s="10"/>
-      <c r="B9" s="10"/>
-      <c r="C9" s="10"/>
-      <c r="D9" s="10"/>
-      <c r="E9" s="11" t="s">
+      <c r="A9" s="8"/>
+      <c r="B9" s="8"/>
+      <c r="C9" s="8"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="F9" s="13">
-        <v>33.566000000000003</v>
-      </c>
-      <c r="G9" s="13">
-        <v>34.405999999999999</v>
-      </c>
-      <c r="H9" s="14"/>
-      <c r="I9" s="14"/>
-      <c r="J9" s="14"/>
-      <c r="K9" s="10"/>
-      <c r="L9" s="10"/>
-      <c r="M9" s="10"/>
-      <c r="N9" s="11" t="s">
+      <c r="F9" s="11">
+        <v>6.71</v>
+      </c>
+      <c r="G9" s="11">
+        <v>9.4190000000000005</v>
+      </c>
+      <c r="H9" s="21">
+        <v>217.042</v>
+      </c>
+      <c r="I9" s="12">
+        <v>295.30099999999999</v>
+      </c>
+      <c r="J9">
+        <v>292.51600000000002</v>
+      </c>
+      <c r="K9" s="8"/>
+      <c r="L9" s="8"/>
+      <c r="M9" s="8"/>
+      <c r="N9" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="O9" s="15">
-        <v>77.754999999999995</v>
-      </c>
-      <c r="P9" s="15">
-        <v>119.75700000000001</v>
-      </c>
-      <c r="Q9" s="15">
-        <v>165.14099999999999</v>
-      </c>
-      <c r="R9" s="15">
-        <v>229.625</v>
-      </c>
-      <c r="S9" s="15">
-        <v>308.29300000000001</v>
+      <c r="O9" s="13">
+        <v>5.4050000000000002</v>
+      </c>
+      <c r="P9" s="13">
+        <v>13.737</v>
+      </c>
+      <c r="Q9" s="13">
+        <v>175.631</v>
+      </c>
+      <c r="R9" s="13">
+        <v>307.55500000000001</v>
+      </c>
+      <c r="S9" s="13">
+        <v>267.93400000000003</v>
       </c>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A10" s="10"/>
-      <c r="B10" s="10"/>
-      <c r="C10" s="10"/>
-      <c r="D10" s="10"/>
-      <c r="E10" s="16" t="s">
+      <c r="A10" s="8"/>
+      <c r="B10" s="8"/>
+      <c r="C10" s="8"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="F10" s="13">
-        <v>31.742000000000001</v>
-      </c>
-      <c r="G10" s="13">
-        <v>38.517000000000003</v>
-      </c>
-      <c r="H10" s="14"/>
-      <c r="I10" s="14"/>
-      <c r="J10" s="14"/>
-      <c r="K10" s="10"/>
-      <c r="L10" s="10"/>
-      <c r="M10" s="10"/>
-      <c r="N10" s="16" t="s">
+      <c r="F10" s="11">
+        <v>7.3369999999999997</v>
+      </c>
+      <c r="G10" s="11">
+        <v>6.6139999999999999</v>
+      </c>
+      <c r="H10" s="21">
+        <v>184.114</v>
+      </c>
+      <c r="I10" s="12">
+        <v>320.28899999999999</v>
+      </c>
+      <c r="J10" s="12">
+        <v>293.92599999999999</v>
+      </c>
+      <c r="K10" s="8"/>
+      <c r="L10" s="8"/>
+      <c r="M10" s="8"/>
+      <c r="N10" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="O10" s="15">
-        <v>76.718999999999994</v>
-      </c>
-      <c r="P10" s="15">
-        <v>99.938999999999993</v>
-      </c>
-      <c r="Q10" s="15">
-        <v>190.42500000000001</v>
-      </c>
-      <c r="R10" s="15">
-        <v>239.77799999999999</v>
-      </c>
-      <c r="S10" s="15">
-        <v>275.48099999999999</v>
+      <c r="O10" s="13">
+        <v>7.016</v>
+      </c>
+      <c r="P10" s="13">
+        <v>11.718</v>
+      </c>
+      <c r="Q10" s="13">
+        <v>199.524</v>
+      </c>
+      <c r="R10" s="13">
+        <v>283.71899999999999</v>
+      </c>
+      <c r="S10" s="13">
+        <v>307.24400000000003</v>
       </c>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A11" s="10"/>
-      <c r="B11" s="10"/>
-      <c r="C11" s="10"/>
-      <c r="D11" s="10"/>
-      <c r="E11" s="16" t="s">
+      <c r="A11" s="8"/>
+      <c r="B11" s="8"/>
+      <c r="C11" s="8"/>
+      <c r="D11" s="8"/>
+      <c r="E11" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="F11" s="13">
-        <v>30.007000000000001</v>
-      </c>
-      <c r="G11" s="13">
-        <v>36.417999999999999</v>
-      </c>
-      <c r="H11" s="14"/>
-      <c r="I11" s="14"/>
-      <c r="J11" s="14"/>
-      <c r="K11" s="10"/>
-      <c r="L11" s="10"/>
-      <c r="M11" s="10"/>
-      <c r="N11" s="16" t="s">
+      <c r="F11" s="11">
+        <v>8.1679999999999993</v>
+      </c>
+      <c r="G11" s="11">
+        <v>7.73</v>
+      </c>
+      <c r="H11" s="12">
+        <v>235.488</v>
+      </c>
+      <c r="I11" s="12">
+        <v>274.56900000000002</v>
+      </c>
+      <c r="J11" s="12">
+        <v>301.834</v>
+      </c>
+      <c r="K11" s="8"/>
+      <c r="L11" s="8"/>
+      <c r="M11" s="8"/>
+      <c r="N11" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="O11" s="15">
-        <v>140.524</v>
-      </c>
-      <c r="P11" s="15">
-        <v>97.105999999999995</v>
-      </c>
-      <c r="Q11" s="15">
-        <v>208.499</v>
-      </c>
-      <c r="R11" s="15">
-        <v>242.53899999999999</v>
-      </c>
-      <c r="S11" s="15">
-        <v>228.61699999999999</v>
+      <c r="O11" s="13">
+        <v>6.44</v>
+      </c>
+      <c r="P11" s="13">
+        <v>11.866</v>
+      </c>
+      <c r="Q11" s="13">
+        <v>208.85300000000001</v>
+      </c>
+      <c r="R11" s="13">
+        <v>292.48099999999999</v>
+      </c>
+      <c r="S11" s="13">
+        <v>305.84800000000001</v>
       </c>
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A12" s="10"/>
-      <c r="B12" s="10"/>
-      <c r="C12" s="10"/>
-      <c r="D12" s="10"/>
-      <c r="E12" s="16" t="s">
+      <c r="A12" s="8"/>
+      <c r="B12" s="8"/>
+      <c r="C12" s="8"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="F12" s="13">
-        <v>33.454000000000001</v>
-      </c>
-      <c r="G12" s="13"/>
-      <c r="H12" s="14"/>
-      <c r="I12" s="14"/>
-      <c r="J12" s="14"/>
-      <c r="K12" s="10"/>
-      <c r="L12" s="10"/>
-      <c r="M12" s="10"/>
-      <c r="N12" s="16" t="s">
+      <c r="F12" s="11">
+        <v>6.3330000000000002</v>
+      </c>
+      <c r="G12" s="11">
+        <v>6.9409999999999998</v>
+      </c>
+      <c r="H12" s="12">
+        <v>203.16</v>
+      </c>
+      <c r="I12" s="12">
+        <v>302.77199999999999</v>
+      </c>
+      <c r="J12" s="12">
+        <v>325.64499999999998</v>
+      </c>
+      <c r="K12" s="8"/>
+      <c r="L12" s="8"/>
+      <c r="M12" s="8"/>
+      <c r="N12" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="O12" s="15">
-        <v>97.156000000000006</v>
-      </c>
-      <c r="P12" s="15">
-        <v>99.393000000000001</v>
-      </c>
-      <c r="Q12" s="15">
-        <v>172.39699999999999</v>
-      </c>
-      <c r="R12" s="15">
-        <v>278.01600000000002</v>
-      </c>
-      <c r="S12" s="15">
-        <v>233.97800000000001</v>
+      <c r="O12" s="13">
+        <v>6.0650000000000004</v>
+      </c>
+      <c r="P12" s="13">
+        <v>13.981</v>
+      </c>
+      <c r="Q12" s="13">
+        <v>221.59800000000001</v>
+      </c>
+      <c r="R12" s="13">
+        <v>290.565</v>
+      </c>
+      <c r="S12" s="13">
+        <v>288.25</v>
       </c>
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A13" s="10"/>
-      <c r="B13" s="10"/>
-      <c r="C13" s="10"/>
-      <c r="D13" s="10"/>
-      <c r="E13" s="16" t="s">
+      <c r="A13" s="8"/>
+      <c r="B13" s="8"/>
+      <c r="C13" s="8"/>
+      <c r="D13" s="8"/>
+      <c r="E13" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="F13" s="13">
-        <v>31.077999999999999</v>
-      </c>
-      <c r="G13" s="13"/>
-      <c r="H13" s="14"/>
-      <c r="I13" s="14"/>
-      <c r="J13" s="14"/>
-      <c r="K13" s="10"/>
-      <c r="L13" s="10"/>
-      <c r="M13" s="10"/>
-      <c r="N13" s="16" t="s">
+      <c r="F13" s="11">
+        <v>6.4509999999999996</v>
+      </c>
+      <c r="G13" s="11">
+        <v>7.1680000000000001</v>
+      </c>
+      <c r="H13" s="12">
+        <v>202.501</v>
+      </c>
+      <c r="I13" s="12">
+        <v>263.51600000000002</v>
+      </c>
+      <c r="J13" s="12">
+        <v>290.48</v>
+      </c>
+      <c r="K13" s="8"/>
+      <c r="L13" s="8"/>
+      <c r="M13" s="8"/>
+      <c r="N13" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="O13" s="15">
-        <v>77.403000000000006</v>
-      </c>
-      <c r="P13" s="15">
-        <v>103.63500000000001</v>
-      </c>
-      <c r="Q13" s="15">
-        <v>159.054</v>
-      </c>
-      <c r="R13" s="15">
-        <v>240.28299999999999</v>
-      </c>
-      <c r="S13" s="15">
-        <v>249.54400000000001</v>
+      <c r="O13" s="13">
+        <v>6.3159999999999998</v>
+      </c>
+      <c r="P13" s="13">
+        <v>12.119</v>
+      </c>
+      <c r="Q13" s="13">
+        <v>203.37200000000001</v>
+      </c>
+      <c r="R13" s="13">
+        <v>265.06299999999999</v>
+      </c>
+      <c r="S13" s="13">
+        <v>282.33</v>
       </c>
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A14" s="10"/>
-      <c r="B14" s="10"/>
-      <c r="C14" s="10"/>
-      <c r="D14" s="10"/>
-      <c r="E14" s="17" t="s">
+      <c r="A14" s="8"/>
+      <c r="B14" s="8"/>
+      <c r="C14" s="8"/>
+      <c r="D14" s="8"/>
+      <c r="E14" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="F14" s="18"/>
-      <c r="G14" s="18"/>
-      <c r="H14" s="18"/>
-      <c r="I14" s="18"/>
-      <c r="J14" s="18"/>
-      <c r="K14" s="10"/>
-      <c r="L14" s="10"/>
-      <c r="M14" s="10"/>
-      <c r="N14" s="17" t="s">
+      <c r="F14" s="16">
+        <f>AVERAGE(F9:F13)</f>
+        <v>6.9998000000000005</v>
+      </c>
+      <c r="G14" s="16">
+        <f t="shared" ref="G14:J14" si="0">AVERAGE(G9:G13)</f>
+        <v>7.5743999999999998</v>
+      </c>
+      <c r="H14" s="16">
+        <f t="shared" si="0"/>
+        <v>208.46100000000001</v>
+      </c>
+      <c r="I14" s="16">
+        <f t="shared" si="0"/>
+        <v>291.2894</v>
+      </c>
+      <c r="J14" s="16">
+        <f t="shared" si="0"/>
+        <v>300.8802</v>
+      </c>
+      <c r="K14" s="8"/>
+      <c r="L14" s="8"/>
+      <c r="M14" s="8"/>
+      <c r="N14" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="O14" s="18">
-        <v>93.911000000000001</v>
-      </c>
-      <c r="P14" s="18">
-        <v>103.96599999999999</v>
-      </c>
-      <c r="Q14" s="18">
-        <v>179.10300000000001</v>
-      </c>
-      <c r="R14" s="18">
-        <v>246.048</v>
-      </c>
-      <c r="S14" s="18">
-        <v>259.18299999999999</v>
+      <c r="O14" s="16">
+        <f t="shared" ref="O14:S14" si="1">AVERAGE(O9:O13)</f>
+        <v>6.2484000000000002</v>
+      </c>
+      <c r="P14" s="16">
+        <f t="shared" si="1"/>
+        <v>12.684200000000001</v>
+      </c>
+      <c r="Q14" s="16">
+        <f t="shared" si="1"/>
+        <v>201.79560000000001</v>
+      </c>
+      <c r="R14" s="16">
+        <f t="shared" si="1"/>
+        <v>287.87659999999994</v>
+      </c>
+      <c r="S14" s="16">
+        <f t="shared" si="1"/>
+        <v>290.32119999999998</v>
       </c>
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A15" s="10"/>
-      <c r="B15" s="10"/>
-      <c r="C15" s="10"/>
-      <c r="D15" s="10"/>
-      <c r="E15" s="10"/>
-      <c r="F15" s="10"/>
-      <c r="G15" s="10"/>
-      <c r="H15" s="10"/>
-      <c r="I15" s="10"/>
-      <c r="J15" s="10"/>
-      <c r="K15" s="10"/>
-      <c r="L15" s="10"/>
-      <c r="M15" s="10"/>
-      <c r="N15" s="10"/>
-      <c r="O15" s="10"/>
-      <c r="P15" s="10"/>
-      <c r="Q15" s="10"/>
-      <c r="R15" s="10"/>
-      <c r="S15" s="10"/>
+      <c r="A15" s="8"/>
+      <c r="B15" s="8"/>
+      <c r="C15" s="8"/>
+      <c r="D15" s="8"/>
+      <c r="E15" s="8"/>
+      <c r="F15" s="8"/>
+      <c r="G15" s="8"/>
+      <c r="H15" s="8"/>
+      <c r="I15" s="8"/>
+      <c r="J15" s="8"/>
+      <c r="K15" s="8"/>
+      <c r="L15" s="8"/>
+      <c r="M15" s="8"/>
+      <c r="N15" s="8"/>
+      <c r="O15" s="8"/>
+      <c r="P15" s="8"/>
+      <c r="Q15" s="8"/>
+      <c r="R15" s="8"/>
+      <c r="S15" s="8"/>
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A16" s="10"/>
-      <c r="B16" s="10"/>
-      <c r="C16" s="10"/>
-      <c r="D16" s="10"/>
-      <c r="E16" s="10"/>
-      <c r="F16" s="10"/>
-      <c r="G16" s="10"/>
-      <c r="H16" s="10"/>
-      <c r="I16" s="10"/>
-      <c r="J16" s="10"/>
-      <c r="K16" s="10"/>
-      <c r="L16" s="10"/>
-      <c r="M16" s="10"/>
-      <c r="N16" s="10"/>
-      <c r="O16" s="10"/>
-      <c r="P16" s="10"/>
-      <c r="Q16" s="10"/>
-      <c r="R16" s="10"/>
-      <c r="S16" s="10"/>
+      <c r="A16" s="8"/>
+      <c r="B16" s="8"/>
+      <c r="C16" s="8"/>
+      <c r="D16" s="8"/>
+      <c r="E16" s="8"/>
+      <c r="F16" s="8"/>
+      <c r="G16" s="8"/>
+      <c r="H16" s="8"/>
+      <c r="I16" s="8"/>
+      <c r="J16" s="8"/>
+      <c r="K16" s="8"/>
+      <c r="L16" s="8"/>
+      <c r="M16" s="8"/>
+      <c r="N16" s="8"/>
+      <c r="O16" s="8"/>
+      <c r="P16" s="8"/>
+      <c r="Q16" s="8"/>
+      <c r="R16" s="8"/>
+      <c r="S16" s="8"/>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A17" s="10"/>
-      <c r="B17" s="10"/>
-      <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="10"/>
-      <c r="F17" s="10"/>
-      <c r="G17" s="10"/>
-      <c r="H17" s="10"/>
-      <c r="I17" s="10"/>
-      <c r="J17" s="10"/>
-      <c r="K17" s="10"/>
-      <c r="L17" s="10"/>
-      <c r="M17" s="10"/>
-      <c r="N17" s="10"/>
-      <c r="O17" s="10"/>
-      <c r="P17" s="10"/>
-      <c r="Q17" s="10"/>
-      <c r="R17" s="10"/>
-      <c r="S17" s="10"/>
+      <c r="A17" s="8"/>
+      <c r="B17" s="8"/>
+      <c r="C17" s="8"/>
+      <c r="D17" s="8"/>
+      <c r="E17" s="8"/>
+      <c r="F17" s="8"/>
+      <c r="G17" s="8"/>
+      <c r="H17" s="8"/>
+      <c r="I17" s="8"/>
+      <c r="J17" s="8"/>
+      <c r="K17" s="8"/>
+      <c r="L17" s="8"/>
+      <c r="M17" s="8"/>
+      <c r="N17" s="8"/>
+      <c r="O17" s="8"/>
+      <c r="P17" s="8"/>
+      <c r="Q17" s="8"/>
+      <c r="R17" s="8"/>
+      <c r="S17" s="8"/>
     </row>
     <row r="18" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A18" s="10"/>
-      <c r="B18" s="10"/>
-      <c r="C18" s="10"/>
-      <c r="D18" s="10"/>
-      <c r="E18" s="10"/>
-      <c r="F18" s="10"/>
-      <c r="G18" s="10"/>
-      <c r="H18" s="10"/>
-      <c r="I18" s="10"/>
-      <c r="J18" s="10"/>
-      <c r="K18" s="10"/>
-      <c r="L18" s="10"/>
-      <c r="M18" s="10"/>
-      <c r="N18" s="10"/>
-      <c r="O18" s="10"/>
-      <c r="P18" s="10"/>
-      <c r="Q18" s="10"/>
-      <c r="R18" s="10"/>
-      <c r="S18" s="10"/>
+      <c r="A18" s="8"/>
+      <c r="B18" s="8"/>
+      <c r="C18" s="8"/>
+      <c r="D18" s="8"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="8"/>
+      <c r="G18" s="8"/>
+      <c r="H18" s="8"/>
+      <c r="I18" s="8"/>
+      <c r="J18" s="8"/>
+      <c r="K18" s="8"/>
+      <c r="L18" s="8"/>
+      <c r="M18" s="8"/>
+      <c r="N18" s="8"/>
+      <c r="O18" s="8"/>
+      <c r="P18" s="8"/>
+      <c r="Q18" s="8"/>
+      <c r="R18" s="8"/>
+      <c r="S18" s="8"/>
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A19" s="10"/>
-      <c r="B19" s="10"/>
-      <c r="C19" s="10"/>
-      <c r="D19" s="10"/>
-      <c r="E19" s="10"/>
-      <c r="F19" s="10"/>
-      <c r="G19" s="10"/>
-      <c r="H19" s="10"/>
-      <c r="I19" s="10"/>
-      <c r="J19" s="10"/>
-      <c r="K19" s="10"/>
-      <c r="L19" s="10"/>
-      <c r="M19" s="10"/>
-      <c r="N19" s="10"/>
-      <c r="O19" s="10"/>
-      <c r="P19" s="10"/>
-      <c r="Q19" s="10"/>
-      <c r="R19" s="10"/>
-      <c r="S19" s="10"/>
+      <c r="A19" s="8"/>
+      <c r="B19" s="8"/>
+      <c r="C19" s="8"/>
+      <c r="D19" s="8"/>
+      <c r="E19" s="8"/>
+      <c r="F19" s="8"/>
+      <c r="G19" s="8"/>
+      <c r="H19" s="8"/>
+      <c r="I19" s="8"/>
+      <c r="J19" s="8"/>
+      <c r="K19" s="8"/>
+      <c r="L19" s="8"/>
+      <c r="M19" s="8"/>
+      <c r="N19" s="8"/>
+      <c r="O19" s="8"/>
+      <c r="P19" s="8"/>
+      <c r="Q19" s="8"/>
+      <c r="R19" s="8"/>
+      <c r="S19" s="8"/>
     </row>
     <row r="20" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A20" s="10"/>
-      <c r="B20" s="10"/>
-      <c r="C20" s="10"/>
-      <c r="D20" s="10"/>
-      <c r="E20" s="10"/>
-      <c r="F20" s="10"/>
-      <c r="G20" s="10"/>
-      <c r="H20" s="10"/>
-      <c r="I20" s="10"/>
-      <c r="J20" s="10"/>
-      <c r="K20" s="10"/>
-      <c r="L20" s="10"/>
-      <c r="M20" s="10"/>
+      <c r="A20" s="8"/>
+      <c r="B20" s="8"/>
+      <c r="C20" s="8"/>
+      <c r="D20" s="8"/>
+      <c r="E20" s="8"/>
+      <c r="F20" s="8"/>
+      <c r="G20" s="8"/>
+      <c r="H20" s="8"/>
+      <c r="I20" s="8"/>
+      <c r="J20" s="8"/>
+      <c r="K20" s="8"/>
+      <c r="L20" s="8"/>
+      <c r="M20" s="8"/>
       <c r="N20" s="20" t="s">
         <v>13</v>
       </c>
@@ -1790,311 +1859,316 @@
       <c r="S20" s="20"/>
     </row>
     <row r="21" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A21" s="10"/>
-      <c r="B21" s="10"/>
-      <c r="C21" s="10"/>
-      <c r="D21" s="10"/>
-      <c r="E21" s="10"/>
-      <c r="F21" s="10"/>
-      <c r="G21" s="10"/>
-      <c r="H21" s="10"/>
-      <c r="I21" s="10"/>
-      <c r="J21" s="10"/>
-      <c r="K21" s="10"/>
-      <c r="L21" s="10"/>
-      <c r="M21" s="10"/>
-      <c r="N21" s="10"/>
-      <c r="O21" s="10"/>
-      <c r="P21" s="10"/>
-      <c r="Q21" s="10"/>
-      <c r="R21" s="10"/>
-      <c r="S21" s="10"/>
+      <c r="A21" s="8"/>
+      <c r="B21" s="8"/>
+      <c r="C21" s="8"/>
+      <c r="D21" s="8"/>
+      <c r="E21" s="8"/>
+      <c r="F21" s="8"/>
+      <c r="G21" s="8"/>
+      <c r="H21" s="8"/>
+      <c r="I21" s="8"/>
+      <c r="J21" s="8"/>
+      <c r="K21" s="8"/>
+      <c r="L21" s="8"/>
+      <c r="M21" s="8"/>
+      <c r="N21" s="8"/>
+      <c r="O21" s="8"/>
+      <c r="P21" s="8"/>
+      <c r="Q21" s="8"/>
+      <c r="R21" s="8"/>
+      <c r="S21" s="8"/>
     </row>
     <row r="22" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A22" s="10"/>
-      <c r="B22" s="10"/>
-      <c r="C22" s="10"/>
-      <c r="D22" s="10"/>
-      <c r="E22" s="10"/>
-      <c r="F22" s="10"/>
-      <c r="G22" s="10"/>
-      <c r="H22" s="10"/>
-      <c r="I22" s="10"/>
-      <c r="J22" s="10"/>
-      <c r="K22" s="10"/>
-      <c r="L22" s="10"/>
-      <c r="M22" s="10"/>
-      <c r="N22" s="10"/>
-      <c r="O22" s="11">
+      <c r="A22" s="8"/>
+      <c r="B22" s="8"/>
+      <c r="C22" s="8"/>
+      <c r="D22" s="8"/>
+      <c r="E22" s="8"/>
+      <c r="F22" s="8"/>
+      <c r="G22" s="8"/>
+      <c r="H22" s="8"/>
+      <c r="I22" s="8"/>
+      <c r="J22" s="8"/>
+      <c r="K22" s="8"/>
+      <c r="L22" s="8"/>
+      <c r="M22" s="8"/>
+      <c r="N22" s="8"/>
+      <c r="O22" s="9">
         <v>100</v>
       </c>
-      <c r="P22" s="12">
+      <c r="P22" s="10">
         <v>1000</v>
       </c>
-      <c r="Q22" s="12">
+      <c r="Q22" s="10">
         <v>10000</v>
       </c>
-      <c r="R22" s="12">
+      <c r="R22" s="10">
         <v>100000</v>
       </c>
-      <c r="S22" s="12">
+      <c r="S22" s="10">
         <v>150000</v>
       </c>
     </row>
     <row r="23" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A23" s="10"/>
-      <c r="B23" s="10"/>
-      <c r="C23" s="10"/>
-      <c r="D23" s="10"/>
-      <c r="E23" s="10"/>
-      <c r="F23" s="10"/>
-      <c r="G23" s="10"/>
-      <c r="H23" s="10"/>
-      <c r="I23" s="10"/>
-      <c r="J23" s="10"/>
-      <c r="K23" s="10"/>
-      <c r="L23" s="10"/>
-      <c r="M23" s="10"/>
-      <c r="N23" s="11" t="s">
+      <c r="A23" s="8"/>
+      <c r="B23" s="8"/>
+      <c r="C23" s="8"/>
+      <c r="D23" s="8"/>
+      <c r="E23" s="8"/>
+      <c r="F23" s="8"/>
+      <c r="G23" s="8"/>
+      <c r="H23" s="8"/>
+      <c r="I23" s="8"/>
+      <c r="J23" s="8"/>
+      <c r="K23" s="8"/>
+      <c r="L23" s="8"/>
+      <c r="M23" s="8"/>
+      <c r="N23" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="O23" s="15">
-        <v>75.866</v>
-      </c>
-      <c r="P23" s="15">
-        <v>130.58199999999999</v>
-      </c>
-      <c r="Q23" s="15">
-        <v>152.541</v>
-      </c>
-      <c r="R23" s="15">
-        <v>249.38900000000001</v>
-      </c>
-      <c r="S23" s="15">
-        <v>232.51900000000001</v>
+      <c r="O23" s="13">
+        <v>6.069</v>
+      </c>
+      <c r="P23" s="13">
+        <v>13.029</v>
+      </c>
+      <c r="Q23" s="13">
+        <v>190.459</v>
+      </c>
+      <c r="R23" s="13">
+        <v>266.09800000000001</v>
+      </c>
+      <c r="S23" s="13">
+        <v>315.65199999999999</v>
       </c>
     </row>
     <row r="24" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A24" s="10"/>
-      <c r="B24" s="10"/>
-      <c r="C24" s="10"/>
-      <c r="D24" s="10"/>
-      <c r="E24" s="10"/>
-      <c r="F24" s="10"/>
-      <c r="G24" s="10"/>
-      <c r="H24" s="10"/>
-      <c r="I24" s="10"/>
-      <c r="J24" s="10"/>
-      <c r="K24" s="10"/>
-      <c r="L24" s="10"/>
-      <c r="M24" s="10"/>
-      <c r="N24" s="16" t="s">
+      <c r="A24" s="8"/>
+      <c r="B24" s="8"/>
+      <c r="C24" s="8"/>
+      <c r="D24" s="8"/>
+      <c r="E24" s="8"/>
+      <c r="F24" s="8"/>
+      <c r="G24" s="8"/>
+      <c r="H24" s="8"/>
+      <c r="I24" s="8"/>
+      <c r="J24" s="8"/>
+      <c r="K24" s="8"/>
+      <c r="L24" s="8"/>
+      <c r="M24" s="8"/>
+      <c r="N24" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="O24" s="15">
-        <v>94.698999999999998</v>
-      </c>
-      <c r="P24" s="15">
-        <v>99.510999999999996</v>
-      </c>
-      <c r="Q24" s="15">
-        <v>184.23699999999999</v>
-      </c>
-      <c r="R24" s="15">
-        <v>255.25399999999999</v>
-      </c>
-      <c r="S24" s="15">
-        <v>265.57600000000002</v>
+      <c r="O24" s="13">
+        <v>5.9429999999999996</v>
+      </c>
+      <c r="P24" s="13">
+        <v>13.57</v>
+      </c>
+      <c r="Q24" s="13">
+        <v>188.482</v>
+      </c>
+      <c r="R24" s="13">
+        <v>280.65699999999998</v>
+      </c>
+      <c r="S24" s="13">
+        <v>284.303</v>
       </c>
     </row>
     <row r="25" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A25" s="10"/>
-      <c r="B25" s="10"/>
-      <c r="C25" s="10"/>
-      <c r="D25" s="10"/>
-      <c r="E25" s="10"/>
-      <c r="F25" s="10"/>
-      <c r="G25" s="10"/>
-      <c r="H25" s="10"/>
-      <c r="I25" s="10"/>
-      <c r="J25" s="10"/>
-      <c r="K25" s="10"/>
-      <c r="L25" s="10"/>
-      <c r="M25" s="10"/>
-      <c r="N25" s="16" t="s">
+      <c r="A25" s="8"/>
+      <c r="B25" s="8"/>
+      <c r="C25" s="8"/>
+      <c r="D25" s="8"/>
+      <c r="E25" s="8"/>
+      <c r="F25" s="8"/>
+      <c r="G25" s="8"/>
+      <c r="H25" s="8"/>
+      <c r="I25" s="8"/>
+      <c r="J25" s="8"/>
+      <c r="K25" s="8"/>
+      <c r="L25" s="8"/>
+      <c r="M25" s="8"/>
+      <c r="N25" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="O25" s="15">
-        <v>102.77</v>
-      </c>
-      <c r="P25" s="15">
-        <v>100.2</v>
-      </c>
-      <c r="Q25" s="15">
-        <v>175.64099999999999</v>
-      </c>
-      <c r="R25" s="15">
-        <v>230.971</v>
-      </c>
-      <c r="S25" s="15">
-        <v>270.988</v>
+      <c r="O25" s="13">
+        <v>5.4669999999999996</v>
+      </c>
+      <c r="P25" s="13">
+        <v>12.115</v>
+      </c>
+      <c r="Q25" s="13">
+        <v>190.93100000000001</v>
+      </c>
+      <c r="R25" s="13">
+        <v>283.52</v>
+      </c>
+      <c r="S25" s="13">
+        <v>280.161</v>
       </c>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A26" s="10"/>
-      <c r="B26" s="10"/>
-      <c r="C26" s="10"/>
-      <c r="D26" s="10"/>
-      <c r="E26" s="10"/>
-      <c r="F26" s="10"/>
-      <c r="G26" s="10"/>
-      <c r="H26" s="10"/>
-      <c r="I26" s="10"/>
-      <c r="J26" s="10"/>
-      <c r="K26" s="10"/>
-      <c r="L26" s="10"/>
-      <c r="M26" s="10"/>
-      <c r="N26" s="16" t="s">
+      <c r="A26" s="8"/>
+      <c r="B26" s="8"/>
+      <c r="C26" s="8"/>
+      <c r="D26" s="8"/>
+      <c r="E26" s="8"/>
+      <c r="F26" s="8"/>
+      <c r="G26" s="8"/>
+      <c r="H26" s="8"/>
+      <c r="I26" s="8"/>
+      <c r="J26" s="8"/>
+      <c r="K26" s="8"/>
+      <c r="L26" s="8"/>
+      <c r="M26" s="8"/>
+      <c r="N26" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="O26" s="15">
-        <v>78.587000000000003</v>
-      </c>
-      <c r="P26" s="15">
-        <v>114.334</v>
-      </c>
-      <c r="Q26" s="15">
-        <v>210.39599999999999</v>
-      </c>
-      <c r="R26" s="15">
-        <v>261.68400000000003</v>
-      </c>
-      <c r="S26" s="15">
-        <v>242.14</v>
+      <c r="O26" s="13">
+        <v>5.4329999999999998</v>
+      </c>
+      <c r="P26" s="13">
+        <v>13.589</v>
+      </c>
+      <c r="Q26" s="13">
+        <v>186.72200000000001</v>
+      </c>
+      <c r="R26" s="13">
+        <v>290.642</v>
+      </c>
+      <c r="S26" s="13">
+        <v>267.197</v>
       </c>
     </row>
     <row r="27" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A27" s="10"/>
-      <c r="B27" s="10"/>
-      <c r="C27" s="10"/>
-      <c r="D27" s="10"/>
-      <c r="E27" s="10"/>
-      <c r="F27" s="10"/>
-      <c r="G27" s="10"/>
-      <c r="H27" s="10"/>
-      <c r="I27" s="10"/>
-      <c r="J27" s="10"/>
-      <c r="K27" s="10"/>
-      <c r="L27" s="10"/>
-      <c r="M27" s="10"/>
-      <c r="N27" s="16" t="s">
+      <c r="A27" s="8"/>
+      <c r="B27" s="8"/>
+      <c r="C27" s="8"/>
+      <c r="D27" s="8"/>
+      <c r="E27" s="8"/>
+      <c r="F27" s="8"/>
+      <c r="G27" s="8"/>
+      <c r="H27" s="8"/>
+      <c r="I27" s="8"/>
+      <c r="J27" s="8"/>
+      <c r="K27" s="8"/>
+      <c r="L27" s="8"/>
+      <c r="M27" s="8"/>
+      <c r="N27" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="O27" s="15">
-        <v>87.555000000000007</v>
-      </c>
-      <c r="P27" s="15">
-        <v>110.733</v>
-      </c>
-      <c r="Q27" s="15">
-        <v>160.60300000000001</v>
-      </c>
-      <c r="R27" s="15">
-        <v>240.37</v>
-      </c>
-      <c r="S27" s="15">
-        <v>245.50899999999999</v>
+      <c r="O27" s="13">
+        <v>11.071999999999999</v>
+      </c>
+      <c r="P27" s="13">
+        <v>14.61</v>
+      </c>
+      <c r="Q27" s="13">
+        <v>233.09</v>
+      </c>
+      <c r="R27" s="13">
+        <v>267.54399999999998</v>
+      </c>
+      <c r="S27" s="13">
+        <v>301.35599999999999</v>
       </c>
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A28" s="10"/>
-      <c r="B28" s="10"/>
-      <c r="C28" s="10"/>
-      <c r="D28" s="10"/>
-      <c r="E28" s="10"/>
-      <c r="F28" s="10"/>
-      <c r="G28" s="10"/>
-      <c r="H28" s="10"/>
-      <c r="I28" s="10"/>
-      <c r="J28" s="10"/>
-      <c r="K28" s="10"/>
-      <c r="L28" s="10"/>
-      <c r="M28" s="10"/>
-      <c r="N28" s="17" t="s">
+      <c r="A28" s="8"/>
+      <c r="B28" s="8"/>
+      <c r="C28" s="8"/>
+      <c r="D28" s="8"/>
+      <c r="E28" s="8"/>
+      <c r="F28" s="8"/>
+      <c r="G28" s="8"/>
+      <c r="H28" s="8"/>
+      <c r="I28" s="8"/>
+      <c r="J28" s="8"/>
+      <c r="K28" s="8"/>
+      <c r="L28" s="8"/>
+      <c r="M28" s="8"/>
+      <c r="N28" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="O28" s="18">
-        <v>87.894999999999996</v>
-      </c>
-      <c r="P28" s="18">
-        <v>111.072</v>
-      </c>
-      <c r="Q28" s="18">
-        <v>176.684</v>
-      </c>
-      <c r="R28" s="18">
-        <v>247.53399999999999</v>
-      </c>
-      <c r="S28" s="18">
-        <v>251.346</v>
+      <c r="O28" s="16">
+        <f t="shared" ref="O28:S28" si="2">AVERAGE(O23:O27)</f>
+        <v>6.7967999999999993</v>
+      </c>
+      <c r="P28" s="16">
+        <f t="shared" si="2"/>
+        <v>13.3826</v>
+      </c>
+      <c r="Q28" s="16">
+        <f t="shared" si="2"/>
+        <v>197.93680000000001</v>
+      </c>
+      <c r="R28" s="16">
+        <f t="shared" si="2"/>
+        <v>277.69219999999996</v>
+      </c>
+      <c r="S28" s="16">
+        <f t="shared" si="2"/>
+        <v>289.73380000000003</v>
       </c>
     </row>
     <row r="29" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A29" s="10"/>
-      <c r="B29" s="10"/>
-      <c r="C29" s="10"/>
-      <c r="D29" s="10"/>
-      <c r="E29" s="10"/>
-      <c r="F29" s="10"/>
-      <c r="G29" s="10"/>
-      <c r="H29" s="10"/>
-      <c r="I29" s="10"/>
-      <c r="J29" s="10"/>
-      <c r="K29" s="10"/>
-      <c r="L29" s="10"/>
-      <c r="M29" s="10"/>
-      <c r="N29" s="10"/>
-      <c r="O29" s="10"/>
-      <c r="P29" s="10"/>
-      <c r="Q29" s="10"/>
-      <c r="R29" s="10"/>
-      <c r="S29" s="10"/>
+      <c r="A29" s="8"/>
+      <c r="B29" s="8"/>
+      <c r="C29" s="8"/>
+      <c r="D29" s="8"/>
+      <c r="E29" s="8"/>
+      <c r="F29" s="8"/>
+      <c r="G29" s="8"/>
+      <c r="H29" s="8"/>
+      <c r="I29" s="8"/>
+      <c r="J29" s="8"/>
+      <c r="K29" s="8"/>
+      <c r="L29" s="8"/>
+      <c r="M29" s="8"/>
+      <c r="N29" s="8"/>
+      <c r="O29" s="8"/>
+      <c r="P29" s="8"/>
+      <c r="Q29" s="8"/>
+      <c r="R29" s="8"/>
+      <c r="S29" s="8"/>
     </row>
     <row r="30" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A30" s="10"/>
-      <c r="B30" s="10"/>
-      <c r="C30" s="10"/>
-      <c r="D30" s="10"/>
-      <c r="E30" s="10"/>
-      <c r="F30" s="10"/>
-      <c r="G30" s="10"/>
-      <c r="H30" s="10"/>
-      <c r="I30" s="10"/>
-      <c r="J30" s="10"/>
-      <c r="K30" s="10"/>
-      <c r="L30" s="10"/>
-      <c r="M30" s="10"/>
-      <c r="N30" s="10"/>
-      <c r="O30" s="10"/>
-      <c r="P30" s="10"/>
-      <c r="Q30" s="10"/>
-      <c r="R30" s="10"/>
-      <c r="S30" s="10"/>
+      <c r="A30" s="8"/>
+      <c r="B30" s="8"/>
+      <c r="C30" s="8"/>
+      <c r="D30" s="8"/>
+      <c r="E30" s="8"/>
+      <c r="F30" s="8"/>
+      <c r="G30" s="8"/>
+      <c r="H30" s="8"/>
+      <c r="I30" s="8"/>
+      <c r="J30" s="8"/>
+      <c r="K30" s="8"/>
+      <c r="L30" s="8"/>
+      <c r="M30" s="8"/>
+      <c r="N30" s="8"/>
+      <c r="O30" s="8"/>
+      <c r="P30" s="8"/>
+      <c r="Q30" s="8"/>
+      <c r="R30" s="8"/>
+      <c r="S30" s="8"/>
     </row>
     <row r="31" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A31" s="10"/>
-      <c r="B31" s="10"/>
-      <c r="C31" s="10"/>
-      <c r="D31" s="10"/>
-      <c r="E31" s="10"/>
-      <c r="F31" s="10"/>
-      <c r="G31" s="10"/>
-      <c r="H31" s="10"/>
-      <c r="I31" s="10"/>
-      <c r="J31" s="10"/>
-      <c r="K31" s="10"/>
-      <c r="L31" s="10"/>
-      <c r="M31" s="10"/>
+      <c r="A31" s="8"/>
+      <c r="B31" s="8"/>
+      <c r="C31" s="8"/>
+      <c r="D31" s="8"/>
+      <c r="E31" s="8"/>
+      <c r="F31" s="8"/>
+      <c r="G31" s="8"/>
+      <c r="H31" s="8"/>
+      <c r="I31" s="8"/>
+      <c r="J31" s="8"/>
+      <c r="K31" s="8"/>
+      <c r="L31" s="8"/>
+      <c r="M31" s="8"/>
       <c r="N31" s="20" t="s">
         <v>14</v>
       </c>
@@ -2105,253 +2179,258 @@
       <c r="S31" s="20"/>
     </row>
     <row r="32" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A32" s="10"/>
-      <c r="B32" s="10"/>
-      <c r="C32" s="10"/>
-      <c r="D32" s="10"/>
-      <c r="E32" s="10"/>
-      <c r="F32" s="10"/>
-      <c r="G32" s="10"/>
-      <c r="H32" s="10"/>
-      <c r="I32" s="10"/>
-      <c r="J32" s="10"/>
-      <c r="K32" s="10"/>
-      <c r="L32" s="10"/>
-      <c r="M32" s="10"/>
-      <c r="N32" s="10"/>
-      <c r="O32" s="10"/>
-      <c r="P32" s="10"/>
-      <c r="Q32" s="10"/>
-      <c r="R32" s="10"/>
-      <c r="S32" s="10"/>
+      <c r="A32" s="8"/>
+      <c r="B32" s="8"/>
+      <c r="C32" s="8"/>
+      <c r="D32" s="8"/>
+      <c r="E32" s="8"/>
+      <c r="F32" s="8"/>
+      <c r="G32" s="8"/>
+      <c r="H32" s="8"/>
+      <c r="I32" s="8"/>
+      <c r="J32" s="8"/>
+      <c r="K32" s="8"/>
+      <c r="L32" s="8"/>
+      <c r="M32" s="8"/>
+      <c r="N32" s="8"/>
+      <c r="O32" s="8"/>
+      <c r="P32" s="8"/>
+      <c r="Q32" s="8"/>
+      <c r="R32" s="8"/>
+      <c r="S32" s="8"/>
     </row>
     <row r="33" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A33" s="10"/>
-      <c r="B33" s="10"/>
-      <c r="C33" s="10"/>
-      <c r="D33" s="10"/>
-      <c r="E33" s="10"/>
-      <c r="F33" s="10"/>
-      <c r="G33" s="10"/>
-      <c r="H33" s="10"/>
-      <c r="I33" s="10"/>
-      <c r="J33" s="10"/>
-      <c r="K33" s="10"/>
-      <c r="L33" s="10"/>
-      <c r="M33" s="10"/>
-      <c r="N33" s="10"/>
-      <c r="O33" s="11">
+      <c r="A33" s="8"/>
+      <c r="B33" s="8"/>
+      <c r="C33" s="8"/>
+      <c r="D33" s="8"/>
+      <c r="E33" s="8"/>
+      <c r="F33" s="8"/>
+      <c r="G33" s="8"/>
+      <c r="H33" s="8"/>
+      <c r="I33" s="8"/>
+      <c r="J33" s="8"/>
+      <c r="K33" s="8"/>
+      <c r="L33" s="8"/>
+      <c r="M33" s="8"/>
+      <c r="N33" s="8"/>
+      <c r="O33" s="9">
         <v>100</v>
       </c>
-      <c r="P33" s="12">
+      <c r="P33" s="10">
         <v>1000</v>
       </c>
-      <c r="Q33" s="12">
+      <c r="Q33" s="10">
         <v>10000</v>
       </c>
-      <c r="R33" s="12">
+      <c r="R33" s="10">
         <v>100000</v>
       </c>
-      <c r="S33" s="12">
+      <c r="S33" s="10">
         <v>150000</v>
       </c>
     </row>
     <row r="34" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A34" s="10"/>
-      <c r="B34" s="10"/>
-      <c r="C34" s="10"/>
-      <c r="D34" s="10"/>
-      <c r="E34" s="10"/>
-      <c r="F34" s="10"/>
-      <c r="G34" s="10"/>
-      <c r="H34" s="10"/>
-      <c r="I34" s="10"/>
-      <c r="J34" s="10"/>
-      <c r="K34" s="10"/>
-      <c r="L34" s="10"/>
-      <c r="M34" s="10"/>
-      <c r="N34" s="11" t="s">
+      <c r="A34" s="8"/>
+      <c r="B34" s="8"/>
+      <c r="C34" s="8"/>
+      <c r="D34" s="8"/>
+      <c r="E34" s="8"/>
+      <c r="F34" s="8"/>
+      <c r="G34" s="8"/>
+      <c r="H34" s="8"/>
+      <c r="I34" s="8"/>
+      <c r="J34" s="8"/>
+      <c r="K34" s="8"/>
+      <c r="L34" s="8"/>
+      <c r="M34" s="8"/>
+      <c r="N34" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="O34" s="15">
-        <v>55.804000000000002</v>
-      </c>
-      <c r="P34" s="15">
-        <v>50.383000000000003</v>
-      </c>
-      <c r="Q34" s="15">
-        <v>51.292999999999999</v>
-      </c>
-      <c r="R34" s="15">
-        <v>52.933999999999997</v>
-      </c>
-      <c r="S34" s="15">
-        <v>52.692999999999998</v>
+      <c r="O34" s="13">
+        <v>3.141</v>
+      </c>
+      <c r="P34" s="13">
+        <v>8.093</v>
+      </c>
+      <c r="Q34" s="13">
+        <v>39.143000000000001</v>
+      </c>
+      <c r="R34" s="13">
+        <v>380.97399999999999</v>
+      </c>
+      <c r="S34" s="13">
+        <v>400.61900000000003</v>
       </c>
     </row>
     <row r="35" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A35" s="10"/>
-      <c r="B35" s="10"/>
-      <c r="C35" s="10"/>
-      <c r="D35" s="10"/>
-      <c r="E35" s="10"/>
-      <c r="F35" s="10"/>
-      <c r="G35" s="10"/>
-      <c r="H35" s="10"/>
-      <c r="I35" s="10"/>
-      <c r="J35" s="10"/>
-      <c r="K35" s="10"/>
-      <c r="L35" s="10"/>
-      <c r="M35" s="10"/>
-      <c r="N35" s="16" t="s">
+      <c r="A35" s="8"/>
+      <c r="B35" s="8"/>
+      <c r="C35" s="8"/>
+      <c r="D35" s="8"/>
+      <c r="E35" s="8"/>
+      <c r="F35" s="8"/>
+      <c r="G35" s="8"/>
+      <c r="H35" s="8"/>
+      <c r="I35" s="8"/>
+      <c r="J35" s="8"/>
+      <c r="K35" s="8"/>
+      <c r="L35" s="8"/>
+      <c r="M35" s="8"/>
+      <c r="N35" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="O35" s="15">
-        <v>65.367999999999995</v>
-      </c>
-      <c r="P35" s="15">
-        <v>69.436999999999998</v>
-      </c>
-      <c r="Q35" s="15">
-        <v>51.094999999999999</v>
-      </c>
-      <c r="R35" s="15">
-        <v>52.177</v>
-      </c>
-      <c r="S35" s="15">
-        <v>58.481000000000002</v>
+      <c r="O35" s="13">
+        <v>3.1739999999999999</v>
+      </c>
+      <c r="P35" s="13">
+        <v>6.7140000000000004</v>
+      </c>
+      <c r="Q35">
+        <v>45.697000000000003</v>
+      </c>
+      <c r="R35" s="13">
+        <v>382.86</v>
+      </c>
+      <c r="S35" s="13">
+        <v>376.42700000000002</v>
       </c>
     </row>
     <row r="36" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A36" s="10"/>
-      <c r="B36" s="10"/>
-      <c r="C36" s="10"/>
-      <c r="D36" s="10"/>
-      <c r="E36" s="10"/>
-      <c r="F36" s="10"/>
-      <c r="G36" s="10"/>
-      <c r="H36" s="10"/>
-      <c r="I36" s="10"/>
-      <c r="J36" s="10"/>
-      <c r="K36" s="10"/>
-      <c r="L36" s="10"/>
-      <c r="M36" s="10"/>
-      <c r="N36" s="16" t="s">
+      <c r="A36" s="8"/>
+      <c r="B36" s="8"/>
+      <c r="C36" s="8"/>
+      <c r="D36" s="8"/>
+      <c r="E36" s="8"/>
+      <c r="F36" s="8"/>
+      <c r="G36" s="8"/>
+      <c r="H36" s="8"/>
+      <c r="I36" s="8"/>
+      <c r="J36" s="8"/>
+      <c r="K36" s="8"/>
+      <c r="L36" s="8"/>
+      <c r="M36" s="8"/>
+      <c r="N36" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="O36" s="15">
-        <v>56.311</v>
-      </c>
-      <c r="P36" s="15">
-        <v>53.951999999999998</v>
-      </c>
-      <c r="Q36" s="15">
-        <v>52.320999999999998</v>
-      </c>
-      <c r="R36" s="15">
-        <v>65.504000000000005</v>
-      </c>
-      <c r="S36" s="15">
-        <v>64.885000000000005</v>
+      <c r="O36" s="13">
+        <v>3.7469999999999999</v>
+      </c>
+      <c r="P36" s="13">
+        <v>6.2389999999999999</v>
+      </c>
+      <c r="Q36" s="13">
+        <v>40.656999999999996</v>
+      </c>
+      <c r="R36" s="22">
+        <v>397.13099999999997</v>
+      </c>
+      <c r="S36" s="13">
+        <v>453.613</v>
       </c>
     </row>
     <row r="37" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A37" s="10"/>
-      <c r="B37" s="10"/>
-      <c r="C37" s="10"/>
-      <c r="D37" s="10"/>
-      <c r="E37" s="10"/>
-      <c r="F37" s="10"/>
-      <c r="G37" s="10"/>
-      <c r="H37" s="10"/>
-      <c r="I37" s="10"/>
-      <c r="J37" s="10"/>
-      <c r="K37" s="10"/>
-      <c r="L37" s="10"/>
-      <c r="M37" s="10"/>
-      <c r="N37" s="16" t="s">
+      <c r="A37" s="8"/>
+      <c r="B37" s="8"/>
+      <c r="C37" s="8"/>
+      <c r="D37" s="8"/>
+      <c r="E37" s="8"/>
+      <c r="F37" s="8"/>
+      <c r="G37" s="8"/>
+      <c r="H37" s="8"/>
+      <c r="I37" s="8"/>
+      <c r="J37" s="8"/>
+      <c r="K37" s="8"/>
+      <c r="L37" s="8"/>
+      <c r="M37" s="8"/>
+      <c r="N37" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="O37" s="15">
-        <v>63.237000000000002</v>
-      </c>
-      <c r="P37" s="15">
-        <v>51.546999999999997</v>
-      </c>
-      <c r="Q37" s="15">
-        <v>53.494</v>
-      </c>
-      <c r="R37" s="15">
-        <v>55.534999999999997</v>
-      </c>
-      <c r="S37" s="15">
-        <v>59.412999999999997</v>
+      <c r="O37" s="13">
+        <v>3.9590000000000001</v>
+      </c>
+      <c r="P37" s="13">
+        <v>6.4</v>
+      </c>
+      <c r="Q37" s="13">
+        <v>43.514000000000003</v>
+      </c>
+      <c r="R37" s="13">
+        <v>475.61900000000003</v>
+      </c>
+      <c r="S37" s="13">
+        <v>435.17399999999998</v>
       </c>
     </row>
     <row r="38" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A38" s="10"/>
-      <c r="B38" s="10"/>
-      <c r="C38" s="10"/>
-      <c r="D38" s="10"/>
-      <c r="E38" s="10"/>
-      <c r="F38" s="10"/>
-      <c r="G38" s="10"/>
-      <c r="H38" s="10"/>
-      <c r="I38" s="10"/>
-      <c r="J38" s="10"/>
-      <c r="K38" s="10"/>
-      <c r="L38" s="10"/>
-      <c r="M38" s="10"/>
-      <c r="N38" s="16" t="s">
+      <c r="A38" s="8"/>
+      <c r="B38" s="8"/>
+      <c r="C38" s="8"/>
+      <c r="D38" s="8"/>
+      <c r="E38" s="8"/>
+      <c r="F38" s="8"/>
+      <c r="G38" s="8"/>
+      <c r="H38" s="8"/>
+      <c r="I38" s="8"/>
+      <c r="J38" s="8"/>
+      <c r="K38" s="8"/>
+      <c r="L38" s="8"/>
+      <c r="M38" s="8"/>
+      <c r="N38" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="O38" s="15">
-        <v>63.16</v>
-      </c>
-      <c r="P38" s="15">
-        <v>53.555</v>
-      </c>
-      <c r="Q38" s="15">
-        <v>58.774999999999999</v>
-      </c>
-      <c r="R38" s="15">
-        <v>50.853999999999999</v>
-      </c>
-      <c r="S38" s="15">
-        <v>55.906999999999996</v>
+      <c r="O38" s="13">
+        <v>2.339</v>
+      </c>
+      <c r="P38" s="13">
+        <v>10.455</v>
+      </c>
+      <c r="Q38" s="13">
+        <v>50.606000000000002</v>
+      </c>
+      <c r="R38" s="13">
+        <v>399.67899999999997</v>
+      </c>
+      <c r="S38" s="13">
+        <v>434.61700000000002</v>
       </c>
     </row>
     <row r="39" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A39" s="10"/>
-      <c r="B39" s="10"/>
-      <c r="C39" s="10"/>
-      <c r="D39" s="10"/>
-      <c r="E39" s="10"/>
-      <c r="F39" s="10"/>
-      <c r="G39" s="10"/>
-      <c r="H39" s="10"/>
-      <c r="I39" s="10"/>
-      <c r="J39" s="10"/>
-      <c r="K39" s="10"/>
-      <c r="L39" s="10"/>
-      <c r="M39" s="10"/>
-      <c r="N39" s="17" t="s">
+      <c r="A39" s="8"/>
+      <c r="B39" s="8"/>
+      <c r="C39" s="8"/>
+      <c r="D39" s="8"/>
+      <c r="E39" s="8"/>
+      <c r="F39" s="8"/>
+      <c r="G39" s="8"/>
+      <c r="H39" s="8"/>
+      <c r="I39" s="8"/>
+      <c r="J39" s="8"/>
+      <c r="K39" s="8"/>
+      <c r="L39" s="8"/>
+      <c r="M39" s="8"/>
+      <c r="N39" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="O39" s="18">
-        <v>60.776000000000003</v>
-      </c>
-      <c r="P39" s="18">
-        <v>55.774999999999999</v>
-      </c>
-      <c r="Q39" s="18">
-        <v>53.396000000000001</v>
-      </c>
-      <c r="R39" s="18">
-        <v>55.401000000000003</v>
-      </c>
-      <c r="S39" s="18">
-        <v>58.276000000000003</v>
+      <c r="O39" s="16">
+        <f t="shared" ref="O39:S39" si="3">AVERAGE(O34:O38)</f>
+        <v>3.2719999999999998</v>
+      </c>
+      <c r="P39" s="16">
+        <f t="shared" si="3"/>
+        <v>7.5801999999999996</v>
+      </c>
+      <c r="Q39" s="16">
+        <f t="shared" si="3"/>
+        <v>43.923400000000001</v>
+      </c>
+      <c r="R39" s="16">
+        <f t="shared" si="3"/>
+        <v>407.25260000000009</v>
+      </c>
+      <c r="S39" s="16">
+        <f t="shared" si="3"/>
+        <v>420.09000000000003</v>
       </c>
     </row>
   </sheetData>
@@ -2363,5 +2442,6 @@
     <mergeCell ref="N31:S31"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>